<commit_message>
Documento del backend con los números del demo de agua real
- Todo el documento recalculado con el demo nuevo (cortes de 92–97 %, tren de
  tres bombas en La Ceiba y siete en Morichal, tanques a escala, cierres de
  un operador real, «antes → con TRIM» −18 %): cada ejemplo corrido con el
  motor, las 125 capturas regeneradas y revisadas, las referencias
  archivo:línea al día.
- Capítulo 1: el caso de P-201B de La Ceiba con el agua real (colchón 1,84 h
  previsto y observado; cierra LC-16 y LC-07; 1.665 bbl/d contra 1.426 en el
  orden de TRIM) y Morichal (10,1 h; 783 bbl/d contra 1.222 parejo).
- Modelo de datos: ejemplos, especificación y Excel regenerados; validar.sh
  detiene y borra el cluster temporal aunque un paso falle, y armar-tablas
  ya no pierde filas de ejemplo en silencio.
- Pantallas: un cambio que redondea a cero se escribe «0 %» (no «−0 %»); el
  ejemplo para pegar la asignación oficial con cifras del demo nuevo.
</commit_message>
<xml_diff>
--- a/docs/backend/modelo-de-datos.xlsx
+++ b/docs/backend/modelo-de-datos.xlsx
@@ -5780,7 +5780,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Medio</t>
+          <t>Llanos</t>
         </is>
       </c>
     </row>
@@ -5866,7 +5866,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Tren de agua con una sola bomba de reinyección, sin respaldo.</t>
+          <t>Tres bombas de agua en paralelo, sin reserva: si para una, se cierran pozos.</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>19180</t>
+          <t>224200</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>20400</t>
+          <t>267750</t>
         </is>
       </c>
     </row>
@@ -7261,7 +7261,7 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>La bomba que mueve el agua no tiene respaldo: si para, el tanque se llena y se cierran los pozos. Es el cuello de botella del campo.</t>
+          <t>El agua (95 % de lo que sale de los pozos) la sacan tres bombas en paralelo, P-201A, B y C, de 90.000 bbl/d de placa; el cabezal de disposición las limita a unos 89.250 cada una. Si para una, las otras dos no alcanzan: el tanque se llena en un par de horas y hay que cerrar parte de los pozos. Es el cuello de botella del campo.</t>
         </is>
       </c>
     </row>
@@ -8241,11 +8241,7 @@
           <t>Texto al pie.</t>
         </is>
       </c>
-      <c r="K59" s="5" t="inlineStr">
-        <is>
-          <t>sin instrumentar</t>
-        </is>
-      </c>
+      <c r="K59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -8286,11 +8282,7 @@
           <t>nivelDe.tag.</t>
         </is>
       </c>
-      <c r="K60" s="5" t="inlineStr">
-        <is>
-          <t>LI-1102</t>
-        </is>
-      </c>
+      <c r="K60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -8331,11 +8323,7 @@
           <t>nivelDe.tope.</t>
         </is>
       </c>
-      <c r="K61" s="5" t="inlineStr">
-        <is>
-          <t>18.5</t>
-        </is>
-      </c>
+      <c r="K61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -8376,11 +8364,7 @@
           <t>Corriente.</t>
         </is>
       </c>
-      <c r="K62" s="5" t="inlineStr">
-        <is>
-          <t>crudo</t>
-        </is>
-      </c>
+      <c r="K62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
@@ -8417,11 +8401,7 @@
           <t>Código del punto de medición oficial, si lo es.</t>
         </is>
       </c>
-      <c r="K63" s="5" t="inlineStr">
-        <is>
-          <t>PMO-02</t>
-        </is>
-      </c>
+      <c r="K63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -13229,7 +13209,7 @@
       </c>
       <c r="K173" s="5" t="inlineStr">
         <is>
-          <t>928</t>
+          <t>10217</t>
         </is>
       </c>
     </row>
@@ -13322,12 +13302,12 @@
       </c>
       <c r="J175" s="5" t="inlineStr">
         <is>
-          <t>Id del evento como lo emite el borde (EP-LC21-261001-01, EV-2011-0909, SV-SE-2-260828).</t>
+          <t>Id del evento como lo emite el borde (EP-LC21-261001-01, EV-2011-0809, SV-SE-2-260828).</t>
         </is>
       </c>
       <c r="K175" s="5" t="inlineStr">
         <is>
-          <t>EP-LC04-260906-65</t>
+          <t>EP-LC04-260906-85</t>
         </is>
       </c>
     </row>
@@ -13564,7 +13544,7 @@
       </c>
       <c r="K180" s="5" t="inlineStr">
         <is>
-          <t>EP-MN07-260214-16</t>
+          <t>EP-MN07-260214-32</t>
         </is>
       </c>
     </row>
@@ -14459,7 +14439,7 @@
       <c r="I200" s="5" t="inlineStr"/>
       <c r="J200" s="5" t="inlineStr">
         <is>
-          <t>Id de la parada (EV-2011-0909).</t>
+          <t>Id de la parada (EV-2011-0809).</t>
         </is>
       </c>
       <c r="K200" s="5" t="inlineStr">
@@ -15131,7 +15111,7 @@
       </c>
       <c r="K215" s="5" t="inlineStr">
         <is>
-          <t>54.5</t>
+          <t>78.2</t>
         </is>
       </c>
     </row>
@@ -15802,7 +15782,7 @@
       </c>
       <c r="K230" s="5" t="inlineStr">
         <is>
-          <t>4332</t>
+          <t>10223</t>
         </is>
       </c>
     </row>
@@ -16960,7 +16940,7 @@
       </c>
       <c r="K256" s="5" t="inlineStr">
         <is>
-          <t>20400</t>
+          <t>89250</t>
         </is>
       </c>
     </row>
@@ -17046,7 +17026,7 @@
       </c>
       <c r="K258" s="5" t="inlineStr">
         <is>
-          <t>El agua no tiene otra salida: los pozos de disposición son su único destino</t>
+          <t>Lo que P-201A y P-201C no absorben no tiene otra salida</t>
         </is>
       </c>
     </row>
@@ -17937,7 +17917,7 @@
       </c>
       <c r="K277" s="5" t="inlineStr">
         <is>
-          <t>61.199999999999996</t>
+          <t>82.45</t>
         </is>
       </c>
     </row>
@@ -17982,7 +17962,7 @@
       </c>
       <c r="K278" s="5" t="inlineStr">
         <is>
-          <t>80.64000000000001</t>
+          <t>108.64000000000001</t>
         </is>
       </c>
     </row>
@@ -18027,7 +18007,7 @@
       </c>
       <c r="K279" s="5" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>63</t>
         </is>
       </c>
     </row>
@@ -18072,7 +18052,7 @@
       </c>
       <c r="K280" s="5" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>121</t>
         </is>
       </c>
     </row>
@@ -20691,7 +20671,7 @@
       </c>
       <c r="K339" s="5" t="inlineStr">
         <is>
-          <t>{"campos":{"ceiba":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":10900,"diferidoMaxBpd":800,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"zarza":{"metas":[{"desde":"2025-10-01","produccionBpd":3050,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":false}},"palmar":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":3250,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"no","bombas":true,"electrosumergibles":false}},"morichal":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":16700,"diferidoMaxBpd":950,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"guacamayo":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":6300,"diferidoMaxBpd":450,"criterioSinCausa":2}],"perfil":{"gas":"consumo","bombas":true,"electrosumergibles":true}}},"empresa":"Operadora de demostración","tanques":[{"id":"TK-AG-CE","aforo":"Certificado de aforo TK-AG-CE · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de La Ceiba","campoId":"ceiba","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":10000},{"id":"TK-AG-MN","aforo":"Certificado de aforo TK-AG-MN · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de Morichal Norte","campoId":"morichal","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":18000},{"id":"TK-AG-GU","aforo":"Certificado de aforo TK-AG-GU · tabla de 1 cm","bomba":"P-201B","nom… [recortado para el Excel: 3427 caracteres]</t>
+          <t>{"campos":{"ceiba":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":10900,"diferidoMaxBpd":800,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"zarza":{"metas":[{"desde":"2025-10-01","produccionBpd":3050,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":false}},"palmar":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":3250,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"no","bombas":true,"electrosumergibles":false}},"morichal":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":16700,"diferidoMaxBpd":950,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"guacamayo":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":6300,"diferidoMaxBpd":450,"criterioSinCausa":2}],"perfil":{"gas":"consumo","bombas":true,"electrosumergibles":true}}},"empresa":"Operadora de demostración","tanques":[{"id":"TK-AG-CE","aforo":"Certificado de aforo TK-AG-CE · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de La Ceiba","campoId":"ceiba","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":30000},{"id":"TK-AG-MN","aforo":"Certificado de aforo TK-AG-MN · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de Morichal Norte","campoId":"morichal","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":60000},{"id":"TK-AG-GU","aforo":"Certificado de aforo TK-AG-GU · tabla de 1 cm","bomba":"P-201B","nom… [recortado para el Excel: 4193 caracteres]</t>
         </is>
       </c>
     </row>
@@ -21664,7 +21644,7 @@
       </c>
       <c r="K360" s="5" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>30000</t>
         </is>
       </c>
     </row>
@@ -22032,7 +22012,7 @@
       </c>
       <c r="K368" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30100</t>
         </is>
       </c>
     </row>
@@ -22073,7 +22053,7 @@
       </c>
       <c r="K369" s="5" t="inlineStr">
         <is>
-          <t>Única bomba del tren de agua</t>
+          <t>P-201A y P-201C en paralelo, con 30.100 bbl/d libres entre las dos: el cabezal de disposición las limita a unos 89.250 cada una</t>
         </is>
       </c>
     </row>
@@ -24443,7 +24423,7 @@
       </c>
       <c r="K423" s="5" t="inlineStr">
         <is>
-          <t>10004146</t>
+          <t>10004149</t>
         </is>
       </c>
     </row>
@@ -24766,7 +24746,7 @@
       </c>
       <c r="K430" s="5" t="inlineStr">
         <is>
-          <t>bomba</t>
+          <t>aislamiento</t>
         </is>
       </c>
     </row>
@@ -24848,7 +24828,7 @@
       </c>
       <c r="K432" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24T21:51:34+00:00</t>
+          <t>2026-09-26T18:46:00+00:00</t>
         </is>
       </c>
     </row>
@@ -25139,7 +25119,7 @@
       </c>
       <c r="K439" s="5" t="inlineStr">
         <is>
-          <t>EV-M2011-260924</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
     </row>
@@ -25270,7 +25250,7 @@
       </c>
       <c r="K442" s="5" t="inlineStr">
         <is>
-          <t>40012053</t>
+          <t>40012056</t>
         </is>
       </c>
     </row>
@@ -25667,7 +25647,7 @@
       </c>
       <c r="K451" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26T12:26:17.357+00:00</t>
+          <t>2026-09-29T10:55:00+00:00</t>
         </is>
       </c>
     </row>
@@ -25798,7 +25778,7 @@
       </c>
       <c r="K454" s="5" t="inlineStr">
         <is>
-          <t>10004146</t>
+          <t>10004149</t>
         </is>
       </c>
     </row>
@@ -25888,7 +25868,7 @@
       </c>
       <c r="K456" s="5" t="inlineStr">
         <is>
-          <t>EV-M2011-260924</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
     </row>
@@ -27215,7 +27195,7 @@
       </c>
       <c r="K486" s="5" t="inlineStr">
         <is>
-          <t>PR-EV-2011-0922</t>
+          <t>PR-EP-LC04-260926-75</t>
         </is>
       </c>
     </row>
@@ -27305,7 +27285,7 @@
       </c>
       <c r="K488" s="5" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-04</t>
         </is>
       </c>
     </row>
@@ -27354,7 +27334,7 @@
       </c>
       <c r="K489" s="5" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
     </row>
@@ -27403,7 +27383,7 @@
       </c>
       <c r="K490" s="5" t="inlineStr">
         <is>
-          <t>rodamientos</t>
+          <t>aislamiento</t>
         </is>
       </c>
     </row>
@@ -27481,7 +27461,7 @@
       </c>
       <c r="K492" s="5" t="inlineStr">
         <is>
-          <t>Revisar aceite de la cámara de empuje y alineación; programar el cambio con el repuesto en mano.</t>
+          <t>Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.</t>
         </is>
       </c>
     </row>
@@ -27522,7 +27502,7 @@
       </c>
       <c r="K493" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20T15:05:00+00:00</t>
+          <t>2026-09-22T18:46:00+00:00</t>
         </is>
       </c>
     </row>
@@ -27567,7 +27547,7 @@
       </c>
       <c r="K494" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21T19:53:00+00:00</t>
+          <t>2026-09-25T04:22:00+00:00</t>
         </is>
       </c>
     </row>
@@ -27612,7 +27592,7 @@
       </c>
       <c r="K495" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23T10:17:00+00:00</t>
+          <t>2026-09-28T09:10:00+00:00</t>
         </is>
       </c>
     </row>
@@ -27706,7 +27686,7 @@
       </c>
       <c r="K497" s="5" t="inlineStr">
         <is>
-          <t>EV-2011-0922</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
     </row>
@@ -27751,7 +27731,7 @@
       </c>
       <c r="K498" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22T15:05:00+00:00</t>
+          <t>2026-09-26T18:46:00+00:00</t>
         </is>
       </c>
     </row>
@@ -27837,7 +27817,7 @@
       </c>
       <c r="K500" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22T15:05:00+00:00</t>
+          <t>2026-09-26T18:46:00+00:00</t>
         </is>
       </c>
     </row>
@@ -30632,7 +30612,7 @@
       </c>
       <c r="K566" s="5" t="inlineStr">
         <is>
-          <t>PR-EP-GU09-260913-93</t>
+          <t>PR-EP-GU09-260913-17</t>
         </is>
       </c>
     </row>
@@ -32664,7 +32644,7 @@
       </c>
       <c r="K614" s="5" t="inlineStr">
         <is>
-          <t>324688</t>
+          <t>338662</t>
         </is>
       </c>
     </row>
@@ -32709,7 +32689,7 @@
       </c>
       <c r="K615" s="5" t="inlineStr">
         <is>
-          <t>335098.09722222236</t>
+          <t>349521.51805555564</t>
         </is>
       </c>
     </row>
@@ -32844,7 +32824,7 @@
       </c>
       <c r="K618" s="5" t="inlineStr">
         <is>
-          <t>0.9689341798460919</t>
+          <t>0.9689303304815998</t>
         </is>
       </c>
     </row>
@@ -33061,7 +33041,7 @@
       </c>
       <c r="K623" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -33200,7 +33180,7 @@
       </c>
       <c r="K626" s="5" t="inlineStr">
         <is>
-          <t>324688</t>
+          <t>338662</t>
         </is>
       </c>
     </row>
@@ -33241,7 +33221,7 @@
       </c>
       <c r="K627" s="5" t="inlineStr">
         <is>
-          <t>346379.4352822801</t>
+          <t>346378.05919221457</t>
         </is>
       </c>
     </row>
@@ -33282,7 +33262,7 @@
       </c>
       <c r="K628" s="5" t="inlineStr">
         <is>
-          <t>21691.435282280087</t>
+          <t>7716.059192214569</t>
         </is>
       </c>
     </row>
@@ -33323,7 +33303,7 @@
       </c>
       <c r="K629" s="5" t="inlineStr">
         <is>
-          <t>21691.43528228031</t>
+          <t>7716.059192214809</t>
         </is>
       </c>
     </row>
@@ -33364,7 +33344,7 @@
       </c>
       <c r="K630" s="5" t="inlineStr">
         <is>
-          <t>-2.219167072325945e-10</t>
+          <t>-2.4010660126805305e-10</t>
         </is>
       </c>
     </row>
@@ -33409,7 +33389,7 @@
       </c>
       <c r="K631" s="5" t="inlineStr">
         <is>
-          <t>3253.715293317683</t>
+          <t>1157.4088799693204</t>
         </is>
       </c>
     </row>
@@ -33495,7 +33475,7 @@
       </c>
       <c r="K633" s="5" t="inlineStr">
         <is>
-          <t>21691.43528228031</t>
+          <t>7716.059192214809</t>
         </is>
       </c>
     </row>
@@ -33659,7 +33639,7 @@
       </c>
       <c r="K637" s="5" t="inlineStr">
         <is>
-          <t>21691.43528228031</t>
+          <t>7716.059192214809</t>
         </is>
       </c>
     </row>
@@ -33700,7 +33680,7 @@
       </c>
       <c r="K638" s="5" t="inlineStr">
         <is>
-          <t>21493.77069097883</t>
+          <t>7476.615648635969</t>
         </is>
       </c>
     </row>
@@ -33741,7 +33721,7 @@
       </c>
       <c r="K639" s="5" t="inlineStr">
         <is>
-          <t>21493.77069097883</t>
+          <t>7476.615648635969</t>
         </is>
       </c>
     </row>
@@ -33864,7 +33844,7 @@
       </c>
       <c r="K642" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>54.995928755535374</t>
         </is>
       </c>
     </row>
@@ -33905,7 +33885,7 @@
       </c>
       <c r="K643" s="5" t="inlineStr">
         <is>
-          <t>93.73766653767919</t>
+          <t>97.77235913550382</t>
         </is>
       </c>
     </row>
@@ -34069,7 +34049,7 @@
       </c>
       <c r="K647" s="5" t="inlineStr">
         <is>
-          <t>1041188.8935494447</t>
+          <t>370370.8412263042</t>
         </is>
       </c>
     </row>
@@ -34327,7 +34307,7 @@
       </c>
       <c r="K653" s="5" t="inlineStr">
         <is>
-          <t>[{'bbl': 20738.85724968679, 'tipo': 'reinyeccion'}, {'bbl': 754.9134412920458, 'tipo': 'electrosumergible'}, {'bbl': 197.66459130147743, 'tipo': 'energia'}]</t>
+          <t>[{'bbl': 6436.065217892938, 'tipo': 'electrosumergible'}, {'bbl': 1040.5504307430315, 'tipo': 'reinyeccion'}, {'bbl': 239.44354357884006, 'tipo': 'energia'}]</t>
         </is>
       </c>
     </row>
@@ -34372,7 +34352,7 @@
       </c>
       <c r="K654" s="5" t="inlineStr">
         <is>
-          <t>[{"bbl":20738.85724968679,"tipo":"reinyeccion","pozos":18,"equipo":"P-201B","partes":[{"bbl":14649.470625413454,"parte":"sello"},{"bbl":6089.386624273328,"parte":"rodamientos"}],"campoId":"ceiba","eventos":2,"tolerancia":3110.8285881692505},{"bbl":216.65435548454434,"tipo":"electrosumergible","pozos":1,"equipo":"LC-16","partes":[{"bbl":216.65435548454434,"parte":"admision"}],"campoId":"ceiba","eventos":2,"tolerancia":32.498159689858475},{"bbl":197.66459130147743,"tipo":"energia","pozos":2,"equipo":"SE-2","partes":[],"campoId":"ceiba","eventos":2,"tolerancia":29.649692535436152},{"bbl":136.11372039771268,"tipo":"electrosumergible","pozos":1,"equipo":"LC-11","partes":[{"bbl":136.11372039771268,"parte":"bomba"}],"campoId":"ceiba","eventos":1,"tolerancia":20.41706519134548},{"bbl":131.4016050772528,"tipo":"electrosumergible","pozos":1,"equipo":"LC-07","partes":[{"bbl":131.4016050772528,"parte":"motor"}],"campoId":"ceiba","eventos":1,"tolerancia":19.71024516785824},{"bbl":94.61103969430506,"tipo":"electrosumergible","pozos":1,"equipo":"LC-14","partes":[{"bbl":66.61960783208463,"parte":"bomba"},{"bbl":27.991431862220434,"parte":"admision"}],"campoId":"ceiba","eventos":2,"tolerancia":14.191668223012627},{"bbl":60.830226107504224,"tipo":"electrosumergible","pozos":1,"equipo":"LC-08","partes":[{"bbl":60.830226107504224,"parte":"admision"}],"campoId":"ceiba","eventos":1,"tolerancia":9.124545888544908},{"bbl":54.85378625653688,"tipo":"electrosumergible","pozos":1,"equipo":"LC-09","parte… [recortado para el Excel: 2212 caracteres]</t>
+          <t>[{"bbl":3677.2278693078233,"tipo":"electrosumergible","pozos":1,"equipo":"LC-11","fallas":1,"partes":[{"bbl":3677.2278693078233,"parte":"aislamiento"}],"campoId":"ceiba","eventos":1,"disparos":0,"tolerancia":551.5841806601529},{"bbl":2125.5969683085755,"tipo":"electrosumergible","pozos":1,"equipo":"LC-04","fallas":1,"partes":[{"bbl":2125.5969683085755,"parte":"aislamiento"}],"campoId":"ceiba","eventos":1,"disparos":0,"tolerancia":318.839545538696},{"bbl":1040.5504307430315,"tipo":"reinyeccion","pozos":2,"equipo":"P-201B","fallas":1,"partes":[{"bbl":1040.5504307430315,"parte":"rodamientos"}],"campoId":"ceiba","eventos":1,"disparos":0,"tolerancia":156.0825658307318},{"bbl":239.44354357884006,"tipo":"energia","pozos":3,"equipo":"SE-2","partes":[],"campoId":"ceiba","eventos":3,"tolerancia":35.91653653227523},{"bbl":216.6534947639708,"tipo":"electrosumergible","pozos":1,"equipo":"LC-16","fallas":0,"partes":[{"bbl":216.6534947639708,"parte":"admision"}],"campoId":"ceiba","eventos":2,"disparos":2,"tolerancia":32.498030581747145},{"bbl":131.4010830472911,"tipo":"electrosumergible","pozos":1,"equipo":"LC-07","fallas":0,"partes":[{"bbl":131.4010830472911,"parte":"motor"}],"campoId":"ceiba","eventos":1,"disparos":1,"tolerancia":19.71016686334648},{"bbl":94.61066382524777,"tipo":"electrosumergible","pozos":1,"equipo":"LC-14","fallas":0,"partes":[{"bbl":66.61934316689045,"parte":"bomba"},{"bbl":27.991320658357328,"parte":"admision"}],"campoId":"ceiba","eventos":2,"disparos":2,"tolerancia"… [recortado para el Excel: 2684 caracteres]</t>
         </is>
       </c>
     </row>
@@ -34417,7 +34397,7 @@
       </c>
       <c r="K655" s="5" t="inlineStr">
         <is>
-          <t>[{"bbl":14649.470625413454,"horas":34.76,"parte":"sello","fallas":1,"equipos":[{"bbl":14649.470625413454,"equipo":"P-201B","campoId":"ceiba"}],"familia":"inyeccion","disparos":0},{"bbl":6089.386624273328,"horas":15.991111111111111,"parte":"rodamientos","fallas":1,"equipos":[{"bbl":6089.386624273328,"equipo":"P-201B","campoId":"ceiba"}],"familia":"inyeccion","disparos":0},{"bbl":395.9845589162674,"horas":12.699999999999998,"parte":"admision","fallas":0,"equipos":[{"bbl":216.65435548454434,"equipo":"LC-16","campoId":"ceiba"},{"bbl":60.830226107504224,"equipo":"LC-08","campoId":"ceiba"},{"bbl":54.85378625653688,"equipo":"LC-09","campoId":"ceiba"},{"bbl":27.991431862220434,"equipo":"LC-14","campoId":"ceiba"},{"bbl":19.93380213745866,"equipo":"LC-02","campoId":"ceiba"},{"bbl":15.720957068002841,"equipo":"LC-12","campoId":"ceiba"}],"familia":"electrosumergible","disparos":7},{"bbl":202.7333282297973,"horas":5.116666666666667,"parte":"bomba","fallas":0,"equipos":[{"bbl":136.11372039771268,"equipo":"LC-11","campoId":"ceiba"},{"bbl":66.61960783208463,"equipo":"LC-14","campoId":"ceiba"}],"familia":"electrosumergible","disparos":2},{"bbl":131.4016050772528,"horas":3.9166666666666665,"parte":"motor","fallas":0,"equipos":[{"bbl":131.4016050772528,"equipo":"LC-07","campoId":"ceiba"}],"familia":"electrosumergible","disparos":1},{"bbl":24.793949068728327,"horas":1.6333333333333333,"parte":"aislamiento","fallas":0,"equipos":[{"bbl":24.793949068728327,"equipo":"LC-01","campoId":"ceiba"}],"fami… [recortado para el Excel: 1539 caracteres]</t>
+          <t>[{'bbl': 5842.061805922908, 'horas': 148.31666666666666, 'parte': 'aislamiento', 'fallas': 2, 'equipos': [{'bbl': 3677.2278693078233, 'equipo': 'LC-11', 'campoId': 'ceiba'}, {'bbl': 2125.5969683085755, 'equipo': 'LC-04', 'campoId': 'ceiba'}, {'bbl': 24.793850567768047, 'equipo': 'LC-01', 'campoId': 'ceiba'}, {'bbl': 14.443117738741348, 'equipo': 'LC-12', 'campoId': 'ceiba'}], 'familia': 'electrosumergible', 'disparos': 2}, {'bbl': 1040.5504307430315, 'horas': 15.991111111111111, 'parte': 'rodamientos', 'fallas': 1, 'equipos': [{'bbl': 1040.5504307430315, 'equipo': 'P-201B', 'campoId': 'ceiba'}], 'familia': 'inyeccion', 'disparos': 0}, {'bbl': 395.9829857558483, 'horas': 12.699999999999998, 'parte': 'admision', 'fallas': 0, 'equipos': [{'bbl': 216.6534947639708, 'equipo': 'LC-16', 'campoId': 'ceiba'}, {'bbl': 60.829984442262884, 'equipo': 'LC-08', 'campoId': 'ceiba'}, {'bbl': 54.85356833438957, 'equipo': 'LC-09', 'campoId': 'ceiba'}, {'bbl': 27.991320658357328, 'equipo': 'LC-14', 'campoId': 'ceiba'}, {'bbl': 19.933722944803744, 'equipo': 'LC-02', 'campoId': 'ceiba'}, {'bbl': 15.720894612063956, 'equipo': 'LC-12', 'campoId': 'ceiba'}], 'familia': 'electrosumergible', 'disparos': 7}, {'bbl': 131.4010830472911, 'horas': 3.9166666666666665, 'parte': 'motor', 'fallas': 0, 'equipos': [{'bbl': 131.4010830472911, 'equipo': 'LC-07', 'campoId': 'ceiba'}], 'familia': 'electrosumergible', 'disparos': 1}, {'bbl': 66.61934316689045, 'horas': 1.9833333333333334, 'parte': 'bomba', 'fallas': 0, 'equipos': [{'bbl': 66.61934316689045, 'equipo': 'LC-14', 'campoId': 'ceiba'}], 'familia': 'electrosumergible', 'disparos': 1}]</t>
         </is>
       </c>
     </row>
@@ -34507,7 +34487,7 @@
       </c>
       <c r="K657" s="5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -34552,7 +34532,7 @@
       </c>
       <c r="K658" s="5" t="inlineStr">
         <is>
-          <t>fa38baaa420730961c4855543e7a4d6d3f086e665341f9534f30d2c21bd205ac</t>
+          <t>9439920a3b191e5defc44bbf5a02780c01f4c477b4232259de355bd618234cb8</t>
         </is>
       </c>
     </row>
@@ -34638,7 +34618,7 @@
       </c>
       <c r="K660" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -34687,7 +34667,7 @@
       </c>
       <c r="K661" s="5" t="inlineStr">
         <is>
-          <t>EP-LC11-260910-79</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
     </row>
@@ -34732,7 +34712,7 @@
       </c>
       <c r="K662" s="5" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -34912,7 +34892,7 @@
       </c>
       <c r="K666" s="5" t="inlineStr">
         <is>
-          <t>2026-09-10T07:03:00+00:00</t>
+          <t>2026-09-27T05:00:00+00:00</t>
         </is>
       </c>
     </row>
@@ -34957,7 +34937,7 @@
       </c>
       <c r="K667" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11T05:00:00+00:00</t>
+          <t>2026-09-28T05:00:00+00:00</t>
         </is>
       </c>
     </row>
@@ -35002,7 +34982,7 @@
       </c>
       <c r="K668" s="5" t="inlineStr">
         <is>
-          <t>21.95</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -35092,7 +35072,7 @@
       </c>
       <c r="K670" s="5" t="inlineStr">
         <is>
-          <t>1097</t>
+          <t>1076</t>
         </is>
       </c>
     </row>
@@ -35137,7 +35117,7 @@
       </c>
       <c r="K671" s="5" t="inlineStr">
         <is>
-          <t>0.9689341798460919</t>
+          <t>0.9689303304815998</t>
         </is>
       </c>
     </row>
@@ -35182,7 +35162,7 @@
       </c>
       <c r="K672" s="5" t="inlineStr">
         <is>
-          <t>972.1296440267092</t>
+          <t>1042.5690355982015</t>
         </is>
       </c>
     </row>
@@ -35395,7 +35375,7 @@
       </c>
       <c r="K677" s="5" t="inlineStr">
         <is>
-          <t>reinyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
     </row>
@@ -35436,7 +35416,7 @@
       </c>
       <c r="K678" s="5" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-11</t>
         </is>
       </c>
     </row>
@@ -35485,7 +35465,7 @@
       </c>
       <c r="K679" s="5" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
     </row>
@@ -35534,7 +35514,7 @@
       </c>
       <c r="K680" s="5" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
     </row>
@@ -35624,7 +35604,7 @@
       </c>
       <c r="K682" s="5" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
     </row>
@@ -35710,7 +35690,7 @@
       </c>
       <c r="K684" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -35902,7 +35882,7 @@
       </c>
       <c r="K688" s="5" t="inlineStr">
         <is>
-          <t>672.3833333333333</t>
+          <t>635.35</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35927,7 @@
       </c>
       <c r="K689" s="5" t="inlineStr">
         <is>
-          <t>31765.538152074274</t>
+          <t>31765.411954508756</t>
         </is>
       </c>
     </row>
@@ -35992,7 +35972,7 @@
       </c>
       <c r="K690" s="5" t="inlineStr">
         <is>
-          <t>2106.2078888922356</t>
+          <t>3677.2278693078233</t>
         </is>
       </c>
     </row>
@@ -36033,7 +36013,7 @@
       </c>
       <c r="K691" s="5" t="inlineStr">
         <is>
-          <t>29659.330263182055</t>
+          <t>28088.184085200945</t>
         </is>
       </c>
     </row>
@@ -36074,7 +36054,7 @@
       </c>
       <c r="K692" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -36250,7 +36230,7 @@
       </c>
       <c r="K696" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -36381,7 +36361,7 @@
       </c>
       <c r="K699" s="5" t="inlineStr">
         <is>
-          <t>0bdcbf1d9fa5fc6420f2410de1af37e9f84cb3384e58d68515450756cff5c411</t>
+          <t>5419eeb481140b47545569f04ef157c614b65495e455f923feaf3d04cbc7f108</t>
         </is>
       </c>
     </row>
@@ -38179,7 +38159,7 @@
       <c r="J749" s="5" t="inlineStr"/>
       <c r="K749" s="5" t="inlineStr">
         <is>
-          <t>[12443, 12582, 12333, 12477, 12570, 12400, 9003, 12422, 12399, 12321, 12491, 12623, 12231, 12245, 12393, 12430, 12379, 12514, 4332, 0, 11010, 12445, 12497, 11866, 11660, 11637, 11480, 11568, 11437, 11752, 11485]</t>
+          <t>[12447, 12586, 12337, 12481, 12574, 12404, 9006, 12426, 12403, 12325, 12495, 12627, 12235, 12249, 12397, 12434, 12383, 12518, 10223, 9723, 11501, 12449, 12502, 11870, 11664, 11641, 11483, 11571, 11441, 11756, 11489]</t>
         </is>
       </c>
     </row>
@@ -38826,7 +38806,7 @@
       <c r="J768" s="5" t="inlineStr"/>
       <c r="K768" s="5" t="inlineStr">
         <is>
-          <t>40012053</t>
+          <t>40012056</t>
         </is>
       </c>
     </row>
@@ -39196,7 +39176,7 @@
       <c r="J778" s="5" t="inlineStr"/>
       <c r="K778" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26T12:26:17.357+00:00</t>
+          <t>2026-09-29T10:55:00+00:00</t>
         </is>
       </c>
     </row>
@@ -39307,7 +39287,7 @@
       <c r="J781" s="5" t="inlineStr"/>
       <c r="K781" s="5" t="inlineStr">
         <is>
-          <t>10004146</t>
+          <t>10004149</t>
         </is>
       </c>
     </row>
@@ -39381,7 +39361,7 @@
       <c r="J783" s="5" t="inlineStr"/>
       <c r="K783" s="5" t="inlineStr">
         <is>
-          <t>EV-2011-0922</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
     </row>
@@ -41104,7 +41084,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Id de la parada (EV-2011-0909).</t>
+          <t>Id de la parada (EV-2011-0809).</t>
         </is>
       </c>
     </row>
@@ -44598,11 +44578,11 @@
     <col width="27" customWidth="1" min="15" max="15"/>
     <col width="27" customWidth="1" min="16" max="16"/>
     <col width="40" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
     <col width="27" customWidth="1" min="19" max="19"/>
     <col width="19" customWidth="1" min="20" max="20"/>
     <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="27" customWidth="1" min="23" max="23"/>
     <col width="34" customWidth="1" min="24" max="24"/>
     <col width="21" customWidth="1" min="25" max="25"/>
@@ -44667,7 +44647,7 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Magdalena Medio</t>
+          <t>Llanos</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -44677,7 +44657,7 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>Tren de agua con una sola bomba de reinyección, sin respaldo.</t>
+          <t>Tres bombas de agua en paralelo, sin reserva: si para una, se cierran pozos.</t>
         </is>
       </c>
     </row>
@@ -45335,7 +45315,7 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Confirmar nivel en los tanques de agua antes de intentar el arranque: si ya están altos, cerrar primero los pozos aguas arriba.</t>
+          <t>Llevar P-201A y P-201C a su caudal máximo y confirmar el nivel del tanque de agua antes de intentar el arranque: si ya está alto, cerrar primero los pozos con menos crudo por barril de agua.</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
@@ -45433,10 +45413,10 @@
         <v>12000</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>19180</v>
+        <v>224200</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>20400</v>
+        <v>267750</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>3850</v>
@@ -45458,7 +45438,7 @@
       </c>
       <c r="L27" s="9" t="inlineStr">
         <is>
-          <t>La bomba que mueve el agua no tiene respaldo: si para, el tanque se llena y se cierran los pozos. Es el cuello de botella del campo.</t>
+          <t>El agua (95 % de lo que sale de los pozos) la sacan tres bombas en paralelo, P-201A, B y C, de 90.000 bbl/d de placa; el cabezal de disposición las limita a unos 89.250 cada una. Si para una, las otras dos no alcanzan: el tanque se llena en un par de horas y hay que cerrar parte de los pozos. Es el cuello de botella del campo.</t>
         </is>
       </c>
     </row>
@@ -45475,10 +45455,10 @@
         <v>7400</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>7600</v>
+        <v>90300</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>13000</v>
+        <v>110000</v>
       </c>
       <c r="F28" s="9" t="n">
         <v>2100</v>
@@ -45517,10 +45497,10 @@
         <v>19500</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>36400</v>
+        <v>580400</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>44000</v>
+        <v>605500</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>9100</v>
@@ -45542,7 +45522,7 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Manda el levantamiento: 41 pozos con bomba electrosumergible. El compresor de gas, sin respaldo, ya cerró pozos cuando paró.</t>
+          <t>Manda el levantamiento: 41 pozos con bomba electrosumergible y 97 % de agua, que sacan siete bombas casi al tope de lo que deja el cabezal de disposición. El compresor de gas, sin respaldo, ya cerró pozos cuando paró.</t>
         </is>
       </c>
     </row>
@@ -45559,10 +45539,10 @@
         <v>3600</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>2400</v>
+        <v>13180</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>5500</v>
+        <v>16000</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>0</v>
@@ -45584,7 +45564,7 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Campo chico de bombeo mecánico, sin tren de gas, con holgura en crudo y agua.</t>
+          <t>Campo chico de bombeo mecánico, sin tren de gas, con holgura en crudo y agua (80 % de agua, que saca una sola bomba de 16.000 bbl/d).</t>
         </is>
       </c>
     </row>
@@ -45601,7 +45581,7 @@
         <v>3400</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>1100</v>
+        <v>1450</v>
       </c>
       <c r="E31" s="9" t="n">
         <v>4000</v>
@@ -45776,7 +45756,7 @@
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
@@ -45785,7 +45765,7 @@
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Bomba de reinyección</t>
+          <t>Bombas de agua</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -46116,35 +46096,27 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>tanques</t>
+          <t>bomba</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>TK-101</t>
+          <t>P-201A</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>TK-101 · respaldo</t>
+          <t>P-201A</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr"/>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>sin instrumentar</t>
-        </is>
-      </c>
+      <c r="G46" s="9" t="inlineStr"/>
       <c r="H46" s="9" t="inlineStr"/>
       <c r="I46" s="9" t="inlineStr"/>
-      <c r="J46" s="9" t="inlineStr">
-        <is>
-          <t>crudo</t>
-        </is>
-      </c>
+      <c r="J46" s="9" t="inlineStr"/>
       <c r="K46" s="9" t="inlineStr"/>
     </row>
     <row r="47">
@@ -46155,46 +46127,32 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>tanques</t>
+          <t>bomba</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>TK-102</t>
+          <t>P-201B</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>TK-102 · PMO-02</t>
+          <t>P-201B</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>TK-102</t>
+          <t>P-201B</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr"/>
-      <c r="H47" s="9" t="inlineStr">
-        <is>
-          <t>LI-1102</t>
-        </is>
-      </c>
-      <c r="I47" s="9" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="J47" s="9" t="inlineStr">
-        <is>
-          <t>crudo</t>
-        </is>
-      </c>
-      <c r="K47" s="9" t="inlineStr">
-        <is>
-          <t>PMO-02</t>
-        </is>
-      </c>
+      <c r="H47" s="9" t="inlineStr"/>
+      <c r="I47" s="9" t="inlineStr"/>
+      <c r="J47" s="9" t="inlineStr"/>
+      <c r="K47" s="9" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -46594,7 +46552,7 @@
       </c>
       <c r="H60" s="9" t="inlineStr">
         <is>
-          <t>{"campo":"ceiba","gateway":{"id":"EPIC-CEIBA-01","serie":"GRVCEI0016","enlace":"starlink","modelo":"GRV-EPIC-PR1","bufferH":48,"firmware":"3.6.2"},"dispositivos":[{"fuente":{"reloj":"el PLC de la batería","endpoint":"https://pi.ceiba.local/piwebapi","protocolo":"pi-web-api"},"nombre":"V-101","metricas":[{"alto":65,"bajo":35,"tipo":"Nivel de interfase","clase":"continua","limite":"35 – 65","nombre":"LI-1012","unidad":"%","cadenciaS":47},{"alto":8,"bajo":null,"tipo":"Presión diferencial","clase":"continua","limite":"&lt; 8","nombre":"PDI-1012","unidad":"psi","cadenciaS":47}]},{"fuente":{"reloj":"el PLC de la batería","endpoint":"https://pi.ceiba.local/piwebapi","protocolo":"pi-web-api"},"nombre":"C-401","metricas":[{"alto":1250,"bajo":1050,"tipo":"Presión de descarga","clase":"continua","limite":"1.050 – 1.250","nombre":"PI-4011","unidad":"psi","cadenciaS":47},{"alto":120,"bajo":null,"tipo":"Temperatura de descarga","clase":"continua","limite":"&lt; 120","nombre":"TI-4011","unidad":"°C","cadenciaS":47}]},{"fuente":{"reloj":"el PLC de la batería","endpoint":"https://pi.ceiba.local/piwebapi","protocolo":"pi-web-api"},"nombre":"H-302","metricas":[{"alto":310,"bajo":280,"tipo":"Temperatura de piel de tubo","clase":"continua","limite":"280 – 310","nombre":"TI-3021","unidad":"°C","cadenciaS":47},{"alto":450,"bajo":null,"tipo":"Temperatura de chimenea","clase":"continua","limite":"&lt; 450","nombre":"TI-3022","unidad":"°C","cadenciaS":47},{"alto":52,"bajo":38,"tipo":"Consumo de gas combustible… [recortado para el Excel: 7245 caracteres]</t>
+          <t>{"campo":"ceiba","gateway":{"id":"EPIC-CEIBA-01","serie":"GRVCEI0016","enlace":"starlink","modelo":"GRV-EPIC-PR1","bufferH":48,"firmware":"3.6.2"},"dispositivos":[{"fuente":{"reloj":"el PLC de la batería","endpoint":"https://pi.ceiba.local/piwebapi","protocolo":"pi-web-api"},"nombre":"V-101","metricas":[{"alto":65,"bajo":35,"tipo":"Nivel de interfase","clase":"continua","limite":"35 – 65","nombre":"LI-1012","unidad":"%","cadenciaS":47},{"alto":8,"bajo":null,"tipo":"Presión diferencial","clase":"continua","limite":"&lt; 8","nombre":"PDI-1012","unidad":"psi","cadenciaS":47}]},{"fuente":{"reloj":"el PLC de la batería","endpoint":"https://pi.ceiba.local/piwebapi","protocolo":"pi-web-api"},"nombre":"C-401","metricas":[{"alto":1250,"bajo":1050,"tipo":"Presión de descarga","clase":"continua","limite":"1.050 – 1.250","nombre":"PI-4011","unidad":"psi","cadenciaS":47},{"alto":120,"bajo":null,"tipo":"Temperatura de descarga","clase":"continua","limite":"&lt; 120","nombre":"TI-4011","unidad":"°C","cadenciaS":47}]},{"fuente":{"reloj":"el PLC de la batería","endpoint":"https://pi.ceiba.local/piwebapi","protocolo":"pi-web-api"},"nombre":"H-302","metricas":[{"alto":310,"bajo":280,"tipo":"Temperatura de piel de tubo","clase":"continua","limite":"280 – 310","nombre":"TI-3021","unidad":"°C","cadenciaS":47},{"alto":450,"bajo":null,"tipo":"Temperatura de chimenea","clase":"continua","limite":"&lt; 450","nombre":"TI-3022","unidad":"°C","cadenciaS":47},{"alto":52,"bajo":38,"tipo":"Consumo de gas combustible… [recortado para el Excel: 7247 caracteres]</t>
         </is>
       </c>
     </row>
@@ -46658,7 +46616,7 @@
       </c>
       <c r="H62" s="9" t="inlineStr">
         <is>
-          <t>{"campo":"morichal","gateway":{"id":"EPIC-MORICHAL-01","serie":"GRVMOR0017","enlace":"starlink","modelo":"GRV-EPIC-PR1","bufferH":48,"firmware":"3.6.2"},"dispositivos":[{"fuente":{"reloj":"el PLC de la batería","endpoint":"plc-morichal.ot.local:502","protocolo":"modbus-tcp"},"nombre":"MPP-301","metricas":[{"alto":60,"bajo":35,"tipo":"Presión de succión","clase":"continua","limite":"35 – 60","nombre":"PT-3011","unidad":"psi","cadenciaS":1},{"alto":75,"bajo":45,"tipo":"Temperatura de succión","clase":"continua","limite":"45 – 75","nombre":"TE-3011","unidad":"°C","cadenciaS":1},{"alto":8,"bajo":null,"tipo":"Caída de presión del filtro","clase":"continua","limite":"&lt; 8","nombre":"PDT-3011","unidad":"psi","cadenciaS":1},{"alto":360,"bajo":320,"tipo":"Presión de descarga","clase":"continua","limite":"320 – 360","nombre":"PT-3012","unidad":"psi","cadenciaS":1},{"alto":90,"bajo":null,"tipo":"Temperatura de descarga","clase":"continua","limite":"&lt; 90","nombre":"TE-3012","unidad":"°C","cadenciaS":1},{"alto":85,"bajo":null,"tipo":"Temperatura de rodamiento","clase":"continua","limite":"&lt; 85","nombre":"TE-3013","unidad":"°C","cadenciaS":1},{"alto":5.5,"bajo":null,"tipo":"Vibración de la bomba","clase":"continua","limite":"&lt; 5,5","nombre":"VT-3013","unidad":"mm/s","cadenciaS":1},{"alto":130,"bajo":null,"tipo":"Temperatura de devanado","clase":"continua","limite":"&lt; 130","nombre":"TE-3014","unidad":"°C","cadenciaS":1},{"alto":85,"bajo":null,"tipo":"Temperatura de rodamiento del motor","cla… [recortado para el Excel: 9668 caracteres]</t>
+          <t>{"campo":"morichal","gateway":{"id":"EPIC-MORICHAL-01","serie":"GRVMOR0017","enlace":"starlink","modelo":"GRV-EPIC-PR1","bufferH":48,"firmware":"3.6.2"},"dispositivos":[{"fuente":{"reloj":"el PLC de la batería","endpoint":"plc-morichal.ot.local:502","protocolo":"modbus-tcp"},"nombre":"MPP-301","metricas":[{"alto":60,"bajo":35,"tipo":"Presión de succión","clase":"continua","limite":"35 – 60","nombre":"PT-3011","unidad":"psi","cadenciaS":1},{"alto":75,"bajo":45,"tipo":"Temperatura de succión","clase":"continua","limite":"45 – 75","nombre":"TE-3011","unidad":"°C","cadenciaS":1},{"alto":8,"bajo":null,"tipo":"Caída de presión del filtro","clase":"continua","limite":"&lt; 8","nombre":"PDT-3011","unidad":"psi","cadenciaS":1},{"alto":360,"bajo":320,"tipo":"Presión de descarga","clase":"continua","limite":"320 – 360","nombre":"PT-3012","unidad":"psi","cadenciaS":1},{"alto":90,"bajo":null,"tipo":"Temperatura de descarga","clase":"continua","limite":"&lt; 90","nombre":"TE-3012","unidad":"°C","cadenciaS":1},{"alto":85,"bajo":null,"tipo":"Temperatura de rodamiento","clase":"continua","limite":"&lt; 85","nombre":"TE-3013","unidad":"°C","cadenciaS":1},{"alto":5.5,"bajo":null,"tipo":"Vibración de la bomba","clase":"continua","limite":"&lt; 5,5","nombre":"VT-3013","unidad":"mm/s","cadenciaS":1},{"alto":130,"bajo":null,"tipo":"Temperatura de devanado","clase":"continua","limite":"&lt; 130","nombre":"TE-3014","unidad":"°C","cadenciaS":1},{"alto":85,"bajo":null,"tipo":"Temperatura de rodamiento del motor","cla… [recortado para el Excel: 9670 caracteres]</t>
         </is>
       </c>
     </row>
@@ -48274,7 +48232,7 @@
         <v>401</v>
       </c>
       <c r="E135" s="9" t="n">
-        <v>928</v>
+        <v>10217</v>
       </c>
       <c r="F135" s="9" t="n">
         <v>59.5</v>
@@ -48300,7 +48258,7 @@
         <v>393</v>
       </c>
       <c r="E136" s="9" t="n">
-        <v>945</v>
+        <v>10404</v>
       </c>
       <c r="F136" s="9" t="n">
         <v>59.5</v>
@@ -48326,7 +48284,7 @@
         <v>393</v>
       </c>
       <c r="E137" s="9" t="n">
-        <v>963</v>
+        <v>10600</v>
       </c>
       <c r="F137" s="9" t="n">
         <v>59.5</v>
@@ -48352,7 +48310,7 @@
         <v>389</v>
       </c>
       <c r="E138" s="9" t="n">
-        <v>952</v>
+        <v>10475</v>
       </c>
       <c r="F138" s="9" t="n">
         <v>59.5</v>
@@ -48378,7 +48336,7 @@
         <v>376</v>
       </c>
       <c r="E139" s="9" t="n">
-        <v>958</v>
+        <v>10543</v>
       </c>
       <c r="F139" s="9" t="n">
         <v>59.5</v>
@@ -48421,7 +48379,7 @@
     <row r="143">
       <c r="A143" s="9" t="inlineStr">
         <is>
-          <t>EP-LC04-260906-65</t>
+          <t>EP-LC04-260906-85</t>
         </is>
       </c>
       <c r="B143" s="9" t="inlineStr">
@@ -48475,7 +48433,7 @@
     <row r="145">
       <c r="A145" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EV-2011-0809</t>
         </is>
       </c>
       <c r="B145" s="9" t="inlineStr">
@@ -48495,7 +48453,7 @@
       </c>
       <c r="E145" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T02:14:00+00:00</t>
+          <t>2026-08-10T02:14:00+00:00</t>
         </is>
       </c>
     </row>
@@ -48615,7 +48573,7 @@
     <row r="151">
       <c r="A151" s="9" t="inlineStr">
         <is>
-          <t>EP-MN07-260214-16</t>
+          <t>EP-MN07-260214-32</t>
         </is>
       </c>
       <c r="B151" s="9" t="inlineStr">
@@ -48713,7 +48671,7 @@
     <row r="153">
       <c r="A153" s="9" t="inlineStr">
         <is>
-          <t>EP-LC04-260906-65</t>
+          <t>EP-LC04-260906-85</t>
         </is>
       </c>
       <c r="B153" s="9" t="inlineStr">
@@ -48805,7 +48763,7 @@
     <row r="155">
       <c r="A155" s="9" t="inlineStr">
         <is>
-          <t>EP-LC16-261002-25</t>
+          <t>EP-LC16-261002-78</t>
         </is>
       </c>
       <c r="B155" s="9" t="inlineStr">
@@ -48825,7 +48783,7 @@
       </c>
       <c r="E155" s="9" t="inlineStr">
         <is>
-          <t>2026-10-02T13:07:00+00:00</t>
+          <t>2026-10-02T10:43:00+00:00</t>
         </is>
       </c>
       <c r="F155" s="9" t="inlineStr"/>
@@ -48842,7 +48800,7 @@
       <c r="I155" s="9" t="inlineStr"/>
       <c r="J155" s="9" t="inlineStr">
         <is>
-          <t>2026-10-02T13:07:00+00:00</t>
+          <t>2026-10-02T10:43:00+00:00</t>
         </is>
       </c>
     </row>
@@ -49318,7 +49276,7 @@
         </is>
       </c>
       <c r="P167" s="9" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
       <c r="Q167" s="9" t="inlineStr">
         <is>
@@ -49435,7 +49393,7 @@
     <row r="170">
       <c r="A170" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-260819</t>
+          <t>EV-2011-0809</t>
         </is>
       </c>
       <c r="B170" s="9" t="inlineStr">
@@ -49455,12 +49413,12 @@
       </c>
       <c r="E170" s="9" t="inlineStr">
         <is>
-          <t>2026-08-19T23:19:23+00:00</t>
+          <t>2026-08-10T02:14:00+00:00</t>
         </is>
       </c>
       <c r="F170" s="9" t="inlineStr">
         <is>
-          <t>2026-08-20T12:34:04+00:00</t>
+          <t>2026-08-11T12:59:36+00:00</t>
         </is>
       </c>
       <c r="G170" s="9" t="n">
@@ -49471,8 +49429,16 @@
           <t>ZS-2011 · marcha → paro</t>
         </is>
       </c>
-      <c r="I170" s="9" t="inlineStr"/>
-      <c r="J170" s="9" t="inlineStr"/>
+      <c r="I170" s="9" t="inlineStr">
+        <is>
+          <t>LSH-2013</t>
+        </is>
+      </c>
+      <c r="J170" s="9" t="inlineStr">
+        <is>
+          <t>fuga de sello detectada</t>
+        </is>
+      </c>
       <c r="K170" s="9" t="inlineStr"/>
       <c r="L170" s="9" t="inlineStr"/>
       <c r="M170" s="9" t="inlineStr"/>
@@ -49483,18 +49449,18 @@
         </is>
       </c>
       <c r="P170" s="9" t="n">
-        <v>47</v>
+        <v>77.3</v>
       </c>
       <c r="Q170" s="9" t="inlineStr">
         <is>
-          <t>2026-08-19T23:19:23+00:00</t>
+          <t>2026-08-10T02:14:00+00:00</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EV-2011-260819</t>
         </is>
       </c>
       <c r="B171" s="9" t="inlineStr">
@@ -49514,12 +49480,12 @@
       </c>
       <c r="E171" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T02:14:00+00:00</t>
+          <t>2026-08-19T23:19:23+00:00</t>
         </is>
       </c>
       <c r="F171" s="9" t="inlineStr">
         <is>
-          <t>2026-09-11T12:59:36+00:00</t>
+          <t>2026-08-20T12:34:04+00:00</t>
         </is>
       </c>
       <c r="G171" s="9" t="n">
@@ -49530,16 +49496,8 @@
           <t>ZS-2011 · marcha → paro</t>
         </is>
       </c>
-      <c r="I171" s="9" t="inlineStr">
-        <is>
-          <t>LSH-2013</t>
-        </is>
-      </c>
-      <c r="J171" s="9" t="inlineStr">
-        <is>
-          <t>fuga de sello detectada</t>
-        </is>
-      </c>
+      <c r="I171" s="9" t="inlineStr"/>
+      <c r="J171" s="9" t="inlineStr"/>
       <c r="K171" s="9" t="inlineStr"/>
       <c r="L171" s="9" t="inlineStr"/>
       <c r="M171" s="9" t="inlineStr"/>
@@ -49550,11 +49508,11 @@
         </is>
       </c>
       <c r="P171" s="9" t="n">
-        <v>52</v>
+        <v>75.7</v>
       </c>
       <c r="Q171" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T02:14:00+00:00</t>
+          <t>2026-08-19T23:19:23+00:00</t>
         </is>
       </c>
     </row>
@@ -49927,7 +49885,7 @@
         </is>
       </c>
       <c r="D191" s="9" t="n">
-        <v>4332</v>
+        <v>10223</v>
       </c>
       <c r="E191" s="9" t="b">
         <v>1</v>
@@ -49960,7 +49918,7 @@
         </is>
       </c>
       <c r="D192" s="9" t="n">
-        <v>0</v>
+        <v>9723</v>
       </c>
       <c r="E192" s="9" t="b">
         <v>1</v>
@@ -49993,7 +49951,7 @@
         </is>
       </c>
       <c r="D193" s="9" t="n">
-        <v>11596</v>
+        <v>11602</v>
       </c>
       <c r="E193" s="9" t="b">
         <v>1</v>
@@ -50059,7 +50017,7 @@
         </is>
       </c>
       <c r="D195" s="9" t="n">
-        <v>3838</v>
+        <v>5836</v>
       </c>
       <c r="E195" s="9" t="b">
         <v>0</v>
@@ -50545,14 +50503,14 @@
         </is>
       </c>
       <c r="G215" s="9" t="n">
-        <v>20400</v>
+        <v>89250</v>
       </c>
       <c r="H215" s="9" t="n">
         <v>1</v>
       </c>
       <c r="I215" s="9" t="inlineStr">
         <is>
-          <t>El agua no tiene otra salida: los pozos de disposición son su único destino</t>
+          <t>Lo que P-201A y P-201C no absorben no tiene otra salida</t>
         </is>
       </c>
     </row>
@@ -50588,7 +50546,7 @@
         </is>
       </c>
       <c r="G216" s="9" t="n">
-        <v>13000</v>
+        <v>50000</v>
       </c>
       <c r="H216" s="9" t="n">
         <v>0</v>
@@ -50631,7 +50589,7 @@
         </is>
       </c>
       <c r="G217" s="9" t="n">
-        <v>22000</v>
+        <v>90000</v>
       </c>
       <c r="H217" s="9" t="n">
         <v>1</v>
@@ -50674,14 +50632,14 @@
         </is>
       </c>
       <c r="G218" s="9" t="n">
-        <v>24000</v>
+        <v>86500</v>
       </c>
       <c r="H218" s="9" t="n">
         <v>1</v>
       </c>
       <c r="I218" s="9" t="inlineStr">
         <is>
-          <t>Lo que P-201A no absorbe no tiene otra salida</t>
+          <t>Lo que las otras seis bombas del tren no absorben no tiene otra salida</t>
         </is>
       </c>
     </row>
@@ -51149,16 +51107,16 @@
         </is>
       </c>
       <c r="F244" s="9" t="n">
-        <v>61.2</v>
+        <v>82.45</v>
       </c>
       <c r="G244" s="9" t="n">
-        <v>80.64000000000001</v>
+        <v>108.64</v>
       </c>
       <c r="H244" s="9" t="n">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="I244" s="9" t="n">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="J244" s="9" t="inlineStr">
         <is>
@@ -52820,7 +52778,7 @@
       </c>
       <c r="H330" s="9" t="inlineStr">
         <is>
-          <t>{"campos":{"ceiba":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":10900,"diferidoMaxBpd":800,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"zarza":{"metas":[{"desde":"2025-10-01","produccionBpd":3050,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":false}},"palmar":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":3250,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"no","bombas":true,"electrosumergibles":false}},"morichal":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":16700,"diferidoMaxBpd":950,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"guacamayo":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":6300,"diferidoMaxBpd":450,"criterioSinCausa":2}],"perfil":{"gas":"consumo","bombas":true,"electrosumergibles":true}}},"empresa":"Operadora de demostración","tanques":[{"id":"TK-AG-CE","aforo":"Certificado de aforo TK-AG-CE · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de La Ceiba","campoId":"ceiba","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":10000},{"id":"TK-AG-MN","aforo":"Certificado de aforo TK-AG-MN · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de Morichal Norte","campoId":"morichal","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":18000},{"id":"TK-AG-GU","aforo":"Certificado de aforo TK-AG-GU · tabla de 1 cm","bomba":"P-201B","nom… [recortado para el Excel: 3427 caracteres]</t>
+          <t>{"campos":{"ceiba":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":10900,"diferidoMaxBpd":800,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"zarza":{"metas":[{"desde":"2025-10-01","produccionBpd":3050,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":false}},"palmar":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":3250,"diferidoMaxBpd":50,"criterioSinCausa":2}],"perfil":{"gas":"no","bombas":true,"electrosumergibles":false}},"morichal":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":16700,"diferidoMaxBpd":950,"criterioSinCausa":2}],"perfil":{"gas":"venta","bombas":true,"electrosumergibles":true}},"guacamayo":{"metas":[{"desde":"2025-10-01","netbackUsd":48,"produccionBpd":6300,"diferidoMaxBpd":450,"criterioSinCausa":2}],"perfil":{"gas":"consumo","bombas":true,"electrosumergibles":true}}},"empresa":"Operadora de demostración","tanques":[{"id":"TK-AG-CE","aforo":"Certificado de aforo TK-AG-CE · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de La Ceiba","campoId":"ceiba","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":30000},{"id":"TK-AG-MN","aforo":"Certificado de aforo TK-AG-MN · tabla de 1 cm","bomba":"P-201B","nombre":"Tanque de agua de Morichal Norte","campoId":"morichal","altoAlto":0.9,"tagNivel":"LT-2012","capacidadBbl":60000},{"id":"TK-AG-GU","aforo":"Certificado de aforo TK-AG-GU · tabla de 1 cm","bomba":"P-201B","nom… [recortado para el Excel: 4193 caracteres]</t>
         </is>
       </c>
     </row>
@@ -53256,7 +53214,7 @@
         </is>
       </c>
       <c r="G354" s="9" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="H354" s="9" t="n">
         <v>0.9</v>
@@ -53300,7 +53258,7 @@
         </is>
       </c>
       <c r="G355" s="9" t="n">
-        <v>8000</v>
+        <v>20000</v>
       </c>
       <c r="H355" s="9" t="n">
         <v>0.9</v>
@@ -53344,7 +53302,7 @@
         </is>
       </c>
       <c r="G356" s="9" t="n">
-        <v>18000</v>
+        <v>60000</v>
       </c>
       <c r="H356" s="9" t="n">
         <v>0.9</v>
@@ -53417,11 +53375,11 @@
         <v>0</v>
       </c>
       <c r="E360" s="9" t="n">
-        <v>0</v>
+        <v>30100</v>
       </c>
       <c r="F360" s="9" t="inlineStr">
         <is>
-          <t>Única bomba del tren de agua</t>
+          <t>P-201A y P-201C en paralelo, con 30.100 bbl/d libres entre las dos: el cabezal de disposición las limita a unos 89.250 cada una</t>
         </is>
       </c>
     </row>
@@ -53443,11 +53401,11 @@
         <v>3</v>
       </c>
       <c r="E361" s="9" t="n">
-        <v>13000</v>
+        <v>50000</v>
       </c>
       <c r="F361" s="9" t="inlineStr">
         <is>
-          <t>Pozo de disposición alterno con capacidad para todo el caudal</t>
+          <t>P-201C de reserva (50.000 bbl/d), alineada al pozo de disposición alterno: toma todo su caudal</t>
         </is>
       </c>
     </row>
@@ -53495,11 +53453,11 @@
         <v>1</v>
       </c>
       <c r="E363" s="9" t="n">
-        <v>15100</v>
+        <v>39500</v>
       </c>
       <c r="F363" s="9" t="inlineStr">
         <is>
-          <t>P-201A en paralelo, con 15.100 bbl/d libres</t>
+          <t>Las otras seis bombas del tren, con 39.500 bbl/d libres entre todas: el cabezal de disposición las limita a unos 86.500 cada una</t>
         </is>
       </c>
     </row>
@@ -53676,7 +53634,7 @@
         </is>
       </c>
       <c r="C370" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D370" s="9" t="inlineStr">
         <is>
@@ -54846,7 +54804,7 @@
     <row r="429">
       <c r="A429" s="9" t="inlineStr">
         <is>
-          <t>10004146</t>
+          <t>10004149</t>
         </is>
       </c>
       <c r="B429" s="9" t="inlineStr">
@@ -54913,12 +54871,12 @@
     <row r="430">
       <c r="A430" s="9" t="inlineStr">
         <is>
-          <t>10004147</t>
+          <t>10004148</t>
         </is>
       </c>
       <c r="B430" s="9" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="C430" s="9" t="inlineStr">
@@ -54928,16 +54886,16 @@
       </c>
       <c r="D430" s="9" t="inlineStr">
         <is>
-          <t>LC-14</t>
+          <t>LC-04</t>
         </is>
       </c>
       <c r="E430" s="9" t="inlineStr">
         <is>
-          <t>El vigía anticipa falla: bomba de fondo de LC-14</t>
+          <t>Aislamiento del motor y del cable: parada de LC-04</t>
         </is>
       </c>
       <c r="F430" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G430" s="9" t="inlineStr">
         <is>
@@ -54946,27 +54904,31 @@
       </c>
       <c r="H430" s="9" t="inlineStr">
         <is>
-          <t>bomba</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="I430" s="9" t="inlineStr"/>
-      <c r="J430" s="9" t="inlineStr"/>
+      <c r="J430" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-26T18:46:00+00:00</t>
+        </is>
+      </c>
       <c r="K430" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L430" s="9" t="inlineStr">
         <is>
-          <t>["Predicción PR-ceiba-LC-14-bomba · ventana hasta el 30 de sept"]</t>
+          <t>["Parada del PLC EP-LC04-260926-75"]</t>
         </is>
       </c>
       <c r="M430" s="9" t="inlineStr">
         <is>
-          <t>2026-09-25T00:38:17.357+00:00</t>
+          <t>2026-09-26T18:49:00+00:00</t>
         </is>
       </c>
       <c r="N430" s="9" t="inlineStr">
         <is>
-          <t>TRIM · predicción del vigía</t>
+          <t>TRIM · desde la parada del PLC</t>
         </is>
       </c>
       <c r="O430" s="9" t="inlineStr"/>
@@ -54975,7 +54937,11 @@
           <t>trim</t>
         </is>
       </c>
-      <c r="Q430" s="9" t="inlineStr"/>
+      <c r="Q430" s="9" t="inlineStr">
+        <is>
+          <t>EP-LC04-260926-75</t>
+        </is>
+      </c>
       <c r="R430" s="9" t="b">
         <v>1</v>
       </c>
@@ -54988,7 +54954,7 @@
     <row r="431">
       <c r="A431" s="9" t="inlineStr">
         <is>
-          <t>10004145</t>
+          <t>10004147</t>
         </is>
       </c>
       <c r="B431" s="9" t="inlineStr">
@@ -54998,28 +54964,36 @@
       </c>
       <c r="C431" s="9" t="inlineStr">
         <is>
-          <t>morichal</t>
+          <t>guacamayo</t>
         </is>
       </c>
       <c r="D431" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>GU-07</t>
         </is>
       </c>
       <c r="E431" s="9" t="inlineStr">
         <is>
-          <t>Parada de P-201B</t>
+          <t>Aislamiento del motor y del cable: parada de GU-07</t>
         </is>
       </c>
       <c r="F431" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G431" s="9" t="inlineStr"/>
-      <c r="H431" s="9" t="inlineStr"/>
+      <c r="G431" s="9" t="inlineStr">
+        <is>
+          <t>electrosumergible</t>
+        </is>
+      </c>
+      <c r="H431" s="9" t="inlineStr">
+        <is>
+          <t>aislamiento</t>
+        </is>
+      </c>
       <c r="I431" s="9" t="inlineStr"/>
       <c r="J431" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T21:51:34+00:00</t>
+          <t>2026-09-26T07:04:00+00:00</t>
         </is>
       </c>
       <c r="K431" s="9" t="b">
@@ -55027,12 +55001,12 @@
       </c>
       <c r="L431" s="9" t="inlineStr">
         <is>
-          <t>["Parada del PLC EV-M2011-260924"]</t>
+          <t>["Parada del PLC EP-GU07-260926-96"]</t>
         </is>
       </c>
       <c r="M431" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T21:54:34+00:00</t>
+          <t>2026-09-26T07:07:00+00:00</t>
         </is>
       </c>
       <c r="N431" s="9" t="inlineStr">
@@ -55048,7 +55022,7 @@
       </c>
       <c r="Q431" s="9" t="inlineStr">
         <is>
-          <t>EV-M2011-260924</t>
+          <t>EP-GU07-260926-96</t>
         </is>
       </c>
       <c r="R431" s="9" t="b">
@@ -55063,7 +55037,7 @@
     <row r="432">
       <c r="A432" s="9" t="inlineStr">
         <is>
-          <t>10004144</t>
+          <t>10004146</t>
         </is>
       </c>
       <c r="B432" s="9" t="inlineStr">
@@ -55073,17 +55047,17 @@
       </c>
       <c r="C432" s="9" t="inlineStr">
         <is>
-          <t>morichal</t>
+          <t>ceiba</t>
         </is>
       </c>
       <c r="D432" s="9" t="inlineStr">
         <is>
-          <t>MPP-301</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="E432" s="9" t="inlineStr">
         <is>
-          <t>Sello mecánico: parada de MPP-301</t>
+          <t>Aislamiento del motor y del cable: parada de LC-11</t>
         </is>
       </c>
       <c r="F432" s="9" t="n">
@@ -55091,18 +55065,18 @@
       </c>
       <c r="G432" s="9" t="inlineStr">
         <is>
-          <t>multifasica</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="H432" s="9" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="I432" s="9" t="inlineStr"/>
       <c r="J432" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T11:23:05+00:00</t>
+          <t>2026-09-26T00:56:00+00:00</t>
         </is>
       </c>
       <c r="K432" s="9" t="b">
@@ -55110,12 +55084,12 @@
       </c>
       <c r="L432" s="9" t="inlineStr">
         <is>
-          <t>["Parada del PLC EV-3016-260924"]</t>
+          <t>["Parada del PLC EP-LC11-260925-40"]</t>
         </is>
       </c>
       <c r="M432" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T11:26:05+00:00</t>
+          <t>2026-09-26T00:59:00+00:00</t>
         </is>
       </c>
       <c r="N432" s="9" t="inlineStr">
@@ -55131,7 +55105,7 @@
       </c>
       <c r="Q432" s="9" t="inlineStr">
         <is>
-          <t>EV-3016-260924</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="R432" s="9" t="b">
@@ -55146,12 +55120,12 @@
     <row r="433">
       <c r="A433" s="9" t="inlineStr">
         <is>
-          <t>10004143</t>
+          <t>10004150</t>
         </is>
       </c>
       <c r="B433" s="9" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="C433" s="9" t="inlineStr">
@@ -55161,49 +55135,45 @@
       </c>
       <c r="D433" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-14</t>
         </is>
       </c>
       <c r="E433" s="9" t="inlineStr">
         <is>
-          <t>Rodamientos: parada de P-201B</t>
+          <t>El vigía anticipa falla: bomba de fondo de LC-14</t>
         </is>
       </c>
       <c r="F433" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G433" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="H433" s="9" t="inlineStr">
         <is>
-          <t>rodamientos</t>
+          <t>bomba</t>
         </is>
       </c>
       <c r="I433" s="9" t="inlineStr"/>
-      <c r="J433" s="9" t="inlineStr">
-        <is>
-          <t>2026-09-22T15:05:00+00:00</t>
-        </is>
-      </c>
+      <c r="J433" s="9" t="inlineStr"/>
       <c r="K433" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L433" s="9" t="inlineStr">
         <is>
-          <t>["Parada del PLC EV-2011-0922"]</t>
+          <t>["Predicción PR-ceiba-LC-14-bomba · ventana hasta el 30 de sept"]</t>
         </is>
       </c>
       <c r="M433" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22T15:08:00+00:00</t>
+          <t>2026-09-25T00:38:17.357+00:00</t>
         </is>
       </c>
       <c r="N433" s="9" t="inlineStr">
         <is>
-          <t>TRIM · desde la parada del PLC</t>
+          <t>TRIM · predicción del vigía</t>
         </is>
       </c>
       <c r="O433" s="9" t="inlineStr"/>
@@ -55212,11 +55182,7 @@
           <t>trim</t>
         </is>
       </c>
-      <c r="Q433" s="9" t="inlineStr">
-        <is>
-          <t>EV-2011-0922</t>
-        </is>
-      </c>
+      <c r="Q433" s="9" t="inlineStr"/>
       <c r="R433" s="9" t="b">
         <v>1</v>
       </c>
@@ -55318,7 +55284,7 @@
     <row r="437">
       <c r="A437" s="9" t="inlineStr">
         <is>
-          <t>40012053</t>
+          <t>40012056</t>
         </is>
       </c>
       <c r="B437" s="9" t="inlineStr">
@@ -55372,7 +55338,7 @@
       </c>
       <c r="M437" s="9" t="inlineStr">
         <is>
-          <t>10004146</t>
+          <t>10004149</t>
         </is>
       </c>
       <c r="N437" s="9" t="n">
@@ -55388,12 +55354,12 @@
     <row r="438">
       <c r="A438" s="9" t="inlineStr">
         <is>
-          <t>40012054</t>
+          <t>40012048</t>
         </is>
       </c>
       <c r="B438" s="9" t="inlineStr">
         <is>
-          <t>PM03</t>
+          <t>PM01</t>
         </is>
       </c>
       <c r="C438" s="9" t="inlineStr">
@@ -55403,12 +55369,12 @@
       </c>
       <c r="D438" s="9" t="inlineStr">
         <is>
-          <t>LC-14</t>
+          <t>LC-04</t>
         </is>
       </c>
       <c r="E438" s="9" t="inlineStr">
         <is>
-          <t>Revisar sólidos y escala; programar tratamiento químico o el cambio de la bomba.</t>
+          <t>Reparar aislamiento del motor y del cable de LC-04</t>
         </is>
       </c>
       <c r="F438" s="9" t="inlineStr">
@@ -55417,21 +55383,21 @@
         </is>
       </c>
       <c r="G438" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H438" s="9" t="inlineStr">
         <is>
-          <t>2026-09-25T02:26:17.357+00:00</t>
+          <t>2026-09-26T19:46:00+00:00</t>
         </is>
       </c>
       <c r="I438" s="9" t="inlineStr">
         <is>
-          <t>2026-09-25T04:26:17.357+00:00</t>
+          <t>2026-09-26T20:46:00+00:00</t>
         </is>
       </c>
       <c r="J438" s="9" t="inlineStr">
         <is>
-          <t>2026-09-26T12:26:17.357+00:00</t>
+          <t>2026-09-29T10:55:00+00:00</t>
         </is>
       </c>
       <c r="K438" s="9" t="inlineStr">
@@ -55446,13 +55412,17 @@
       </c>
       <c r="M438" s="9" t="inlineStr">
         <is>
-          <t>10004147</t>
+          <t>10004148</t>
         </is>
       </c>
       <c r="N438" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="O438" s="9" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="O438" s="9" t="inlineStr">
+        <is>
+          <t>EP-LC04-260926-75</t>
+        </is>
+      </c>
       <c r="P438" s="9" t="inlineStr">
         <is>
           <t>2026-10-02T19:00:00+00:00</t>
@@ -55462,7 +55432,7 @@
     <row r="439">
       <c r="A439" s="9" t="inlineStr">
         <is>
-          <t>40012045</t>
+          <t>40012047</t>
         </is>
       </c>
       <c r="B439" s="9" t="inlineStr">
@@ -55472,17 +55442,17 @@
       </c>
       <c r="C439" s="9" t="inlineStr">
         <is>
-          <t>morichal</t>
+          <t>guacamayo</t>
         </is>
       </c>
       <c r="D439" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>GU-07</t>
         </is>
       </c>
       <c r="E439" s="9" t="inlineStr">
         <is>
-          <t>Revisar y reparar P-201B</t>
+          <t>Reparar aislamiento del motor y del cable de GU-07</t>
         </is>
       </c>
       <c r="F439" s="9" t="inlineStr">
@@ -55495,17 +55465,17 @@
       </c>
       <c r="H439" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T22:51:34+00:00</t>
+          <t>2026-09-26T08:04:00+00:00</t>
         </is>
       </c>
       <c r="I439" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T23:51:34+00:00</t>
+          <t>2026-09-26T09:04:00+00:00</t>
         </is>
       </c>
       <c r="J439" s="9" t="inlineStr">
         <is>
-          <t>2026-09-28T14:53:06+00:00</t>
+          <t>2026-09-28T22:47:00+00:00</t>
         </is>
       </c>
       <c r="K439" s="9" t="inlineStr"/>
@@ -55516,7 +55486,7 @@
       </c>
       <c r="M439" s="9" t="inlineStr">
         <is>
-          <t>10004145</t>
+          <t>10004147</t>
         </is>
       </c>
       <c r="N439" s="9" t="n">
@@ -55524,7 +55494,7 @@
       </c>
       <c r="O439" s="9" t="inlineStr">
         <is>
-          <t>EV-M2011-260924</t>
+          <t>EP-GU07-260926-96</t>
         </is>
       </c>
       <c r="P439" s="9" t="inlineStr">
@@ -55536,7 +55506,7 @@
     <row r="440">
       <c r="A440" s="9" t="inlineStr">
         <is>
-          <t>40012044</t>
+          <t>40012046</t>
         </is>
       </c>
       <c r="B440" s="9" t="inlineStr">
@@ -55546,17 +55516,17 @@
       </c>
       <c r="C440" s="9" t="inlineStr">
         <is>
-          <t>morichal</t>
+          <t>ceiba</t>
         </is>
       </c>
       <c r="D440" s="9" t="inlineStr">
         <is>
-          <t>MPP-301</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="E440" s="9" t="inlineStr">
         <is>
-          <t>Reparar sello mecánico de MPP-301</t>
+          <t>Reparar aislamiento del motor y del cable de LC-11</t>
         </is>
       </c>
       <c r="F440" s="9" t="inlineStr">
@@ -55569,28 +55539,32 @@
       </c>
       <c r="H440" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T12:23:05+00:00</t>
+          <t>2026-09-26T01:56:00+00:00</t>
         </is>
       </c>
       <c r="I440" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T13:23:05+00:00</t>
+          <t>2026-09-26T02:56:00+00:00</t>
         </is>
       </c>
       <c r="J440" s="9" t="inlineStr">
         <is>
-          <t>2026-09-26T11:47:15+00:00</t>
-        </is>
-      </c>
-      <c r="K440" s="9" t="inlineStr"/>
+          <t>2026-09-29T16:35:00+00:00</t>
+        </is>
+      </c>
+      <c r="K440" s="9" t="inlineStr">
+        <is>
+          <t>tec</t>
+        </is>
+      </c>
       <c r="L440" s="9" t="inlineStr">
         <is>
-          <t>MEC-CONTRATISTA</t>
+          <t>MEC-CEIBA</t>
         </is>
       </c>
       <c r="M440" s="9" t="inlineStr">
         <is>
-          <t>10004144</t>
+          <t>10004146</t>
         </is>
       </c>
       <c r="N440" s="9" t="n">
@@ -55598,7 +55572,7 @@
       </c>
       <c r="O440" s="9" t="inlineStr">
         <is>
-          <t>EV-3016-260924</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="P440" s="9" t="inlineStr">
@@ -55610,12 +55584,12 @@
     <row r="441">
       <c r="A441" s="9" t="inlineStr">
         <is>
-          <t>40012043</t>
+          <t>40012057</t>
         </is>
       </c>
       <c r="B441" s="9" t="inlineStr">
         <is>
-          <t>PM01</t>
+          <t>PM03</t>
         </is>
       </c>
       <c r="C441" s="9" t="inlineStr">
@@ -55625,12 +55599,12 @@
       </c>
       <c r="D441" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-14</t>
         </is>
       </c>
       <c r="E441" s="9" t="inlineStr">
         <is>
-          <t>Reparar rodamientos de P-201B</t>
+          <t>Revisar sólidos y escala; programar tratamiento químico o el cambio de la bomba.</t>
         </is>
       </c>
       <c r="F441" s="9" t="inlineStr">
@@ -55639,21 +55613,21 @@
         </is>
       </c>
       <c r="G441" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H441" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22T16:05:00+00:00</t>
+          <t>2026-09-25T02:26:17.357+00:00</t>
         </is>
       </c>
       <c r="I441" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22T17:05:00+00:00</t>
+          <t>2026-09-25T04:26:17.357+00:00</t>
         </is>
       </c>
       <c r="J441" s="9" t="inlineStr">
         <is>
-          <t>2026-09-23T10:04:28+00:00</t>
+          <t>2026-09-26T12:26:17.357+00:00</t>
         </is>
       </c>
       <c r="K441" s="9" t="inlineStr">
@@ -55668,17 +55642,13 @@
       </c>
       <c r="M441" s="9" t="inlineStr">
         <is>
-          <t>10004143</t>
+          <t>10004150</t>
         </is>
       </c>
       <c r="N441" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="O441" s="9" t="inlineStr">
-        <is>
-          <t>EV-2011-0922</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="O441" s="9" t="inlineStr"/>
       <c r="P441" s="9" t="inlineStr">
         <is>
           <t>2026-10-02T19:00:00+00:00</t>
@@ -56455,7 +56425,7 @@
     <row r="485">
       <c r="A485" s="9" t="inlineStr">
         <is>
-          <t>PR-EV-2011-0922</t>
+          <t>PR-EP-LC04-260926-75</t>
         </is>
       </c>
       <c r="B485" s="9" t="inlineStr">
@@ -56465,38 +56435,38 @@
       </c>
       <c r="C485" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-04</t>
         </is>
       </c>
       <c r="D485" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="E485" s="9" t="inlineStr">
         <is>
-          <t>rodamientos</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="F485" s="9" t="inlineStr"/>
       <c r="G485" s="9" t="inlineStr">
         <is>
-          <t>Revisar aceite de la cámara de empuje y alineación; programar el cambio con el repuesto en mano.</t>
+          <t>Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.</t>
         </is>
       </c>
       <c r="H485" s="9" t="inlineStr">
         <is>
-          <t>2026-09-20T15:05:00+00:00</t>
+          <t>2026-09-22T18:46:00+00:00</t>
         </is>
       </c>
       <c r="I485" s="9" t="inlineStr">
         <is>
-          <t>2026-09-21T19:53:00+00:00</t>
+          <t>2026-09-25T04:22:00+00:00</t>
         </is>
       </c>
       <c r="J485" s="9" t="inlineStr">
         <is>
-          <t>2026-09-23T10:17:00+00:00</t>
+          <t>2026-09-28T09:10:00+00:00</t>
         </is>
       </c>
       <c r="K485" s="9" t="inlineStr">
@@ -56506,66 +56476,66 @@
       </c>
       <c r="L485" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0922</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
       <c r="M485" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22T15:05:00+00:00</t>
+          <t>2026-09-26T18:46:00+00:00</t>
         </is>
       </c>
       <c r="N485" s="9" t="inlineStr"/>
       <c r="O485" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22T15:05:00+00:00</t>
+          <t>2026-09-26T18:46:00+00:00</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="9" t="inlineStr">
         <is>
-          <t>PR-EP-GU09-260913-93</t>
+          <t>PR-EV-2011-0922</t>
         </is>
       </c>
       <c r="B486" s="9" t="inlineStr">
         <is>
-          <t>guacamayo</t>
+          <t>ceiba</t>
         </is>
       </c>
       <c r="C486" s="9" t="inlineStr">
         <is>
-          <t>GU-09</t>
+          <t>P-201B</t>
         </is>
       </c>
       <c r="D486" s="9" t="inlineStr">
         <is>
-          <t>electrosumergible</t>
+          <t>inyeccion</t>
         </is>
       </c>
       <c r="E486" s="9" t="inlineStr">
         <is>
-          <t>aislamiento</t>
+          <t>rodamientos</t>
         </is>
       </c>
       <c r="F486" s="9" t="inlineStr"/>
       <c r="G486" s="9" t="inlineStr">
         <is>
-          <t>Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.</t>
+          <t>Revisar aceite de la cámara de empuje y alineación; programar el cambio con el repuesto en mano.</t>
         </is>
       </c>
       <c r="H486" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T22:23:00+00:00</t>
+          <t>2026-09-20T15:05:00+00:00</t>
         </is>
       </c>
       <c r="I486" s="9" t="inlineStr">
         <is>
-          <t>2026-09-12T17:35:00+00:00</t>
+          <t>2026-09-21T19:53:00+00:00</t>
         </is>
       </c>
       <c r="J486" s="9" t="inlineStr">
         <is>
-          <t>2026-09-15T03:11:00+00:00</t>
+          <t>2026-09-23T10:17:00+00:00</t>
         </is>
       </c>
       <c r="K486" s="9" t="inlineStr">
@@ -56575,25 +56545,25 @@
       </c>
       <c r="L486" s="9" t="inlineStr">
         <is>
-          <t>EP-GU09-260913-93</t>
+          <t>EV-2011-0922</t>
         </is>
       </c>
       <c r="M486" s="9" t="inlineStr">
         <is>
-          <t>2026-09-13T22:23:00+00:00</t>
+          <t>2026-09-22T15:05:00+00:00</t>
         </is>
       </c>
       <c r="N486" s="9" t="inlineStr"/>
       <c r="O486" s="9" t="inlineStr">
         <is>
-          <t>2026-09-13T22:23:00+00:00</t>
+          <t>2026-09-22T15:05:00+00:00</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="9" t="inlineStr">
         <is>
-          <t>PR-EV-2011-0909</t>
+          <t>PR-EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="B487" s="9" t="inlineStr">
@@ -56603,38 +56573,38 @@
       </c>
       <c r="C487" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="D487" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="E487" s="9" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="F487" s="9" t="inlineStr"/>
       <c r="G487" s="9" t="inlineStr">
         <is>
-          <t>Corregir la succión y revisar el plan de sello; tener el cartucho de repuesto en sitio antes de que la fuga crezca.</t>
+          <t>Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.</t>
         </is>
       </c>
       <c r="H487" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05T02:14:00+00:00</t>
+          <t>2026-09-18T00:56:00+00:00</t>
         </is>
       </c>
       <c r="I487" s="9" t="inlineStr">
         <is>
-          <t>2026-09-08T02:14:00+00:00</t>
+          <t>2026-09-22T20:08:00+00:00</t>
         </is>
       </c>
       <c r="J487" s="9" t="inlineStr">
         <is>
-          <t>2026-09-12T02:14:00+00:00</t>
+          <t>2026-09-29T05:44:00+00:00</t>
         </is>
       </c>
       <c r="K487" s="9" t="inlineStr">
@@ -56644,25 +56614,25 @@
       </c>
       <c r="L487" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="M487" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T02:14:00+00:00</t>
+          <t>2026-09-26T00:56:00+00:00</t>
         </is>
       </c>
       <c r="N487" s="9" t="inlineStr"/>
       <c r="O487" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T02:14:00+00:00</t>
+          <t>2026-09-26T00:56:00+00:00</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="9" t="inlineStr">
         <is>
-          <t>PR-morichal-MN-41-aislamiento</t>
+          <t>PR-EP-MN33-260917-72</t>
         </is>
       </c>
       <c r="B488" s="9" t="inlineStr">
@@ -56672,7 +56642,7 @@
       </c>
       <c r="C488" s="9" t="inlineStr">
         <is>
-          <t>MN-41</t>
+          <t>MN-33</t>
         </is>
       </c>
       <c r="D488" s="9" t="inlineStr">
@@ -56693,17 +56663,17 @@
       </c>
       <c r="H488" s="9" t="inlineStr">
         <is>
-          <t>2026-09-03T06:55:34.097+00:00</t>
+          <t>2026-09-13T07:26:00+00:00</t>
         </is>
       </c>
       <c r="I488" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05T02:07:34.097+00:00</t>
+          <t>2026-09-15T17:02:00+00:00</t>
         </is>
       </c>
       <c r="J488" s="9" t="inlineStr">
         <is>
-          <t>2026-09-07T11:43:34.097+00:00</t>
+          <t>2026-09-18T21:50:00+00:00</t>
         </is>
       </c>
       <c r="K488" s="9" t="inlineStr">
@@ -56713,35 +56683,35 @@
       </c>
       <c r="L488" s="9" t="inlineStr">
         <is>
-          <t>EP-MN41-260903-06</t>
+          <t>EP-MN33-260917-72</t>
         </is>
       </c>
       <c r="M488" s="9" t="inlineStr">
         <is>
-          <t>2026-09-03T11:40:00+00:00</t>
+          <t>2026-09-17T07:26:00+00:00</t>
         </is>
       </c>
       <c r="N488" s="9" t="inlineStr"/>
       <c r="O488" s="9" t="inlineStr">
         <is>
-          <t>2026-09-03T11:40:00+00:00</t>
+          <t>2026-09-17T07:26:00+00:00</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="9" t="inlineStr">
         <is>
-          <t>PR-EP-MN23-260905-57</t>
+          <t>PR-EP-GU09-260913-17</t>
         </is>
       </c>
       <c r="B489" s="9" t="inlineStr">
         <is>
-          <t>morichal</t>
+          <t>guacamayo</t>
         </is>
       </c>
       <c r="C489" s="9" t="inlineStr">
         <is>
-          <t>MN-23</t>
+          <t>GU-09</t>
         </is>
       </c>
       <c r="D489" s="9" t="inlineStr">
@@ -56751,28 +56721,28 @@
       </c>
       <c r="E489" s="9" t="inlineStr">
         <is>
-          <t>admision</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="F489" s="9" t="inlineStr"/>
       <c r="G489" s="9" t="inlineStr">
         <is>
-          <t>Bajar la frecuencia o revisar el nivel de fluido antes de que dispare por baja carga.</t>
+          <t>Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.</t>
         </is>
       </c>
       <c r="H489" s="9" t="inlineStr">
         <is>
-          <t>2026-09-01T19:17:00+00:00</t>
+          <t>2026-09-07T22:23:00+00:00</t>
         </is>
       </c>
       <c r="I489" s="9" t="inlineStr">
         <is>
-          <t>2026-09-04T04:53:00+00:00</t>
+          <t>2026-09-11T12:47:00+00:00</t>
         </is>
       </c>
       <c r="J489" s="9" t="inlineStr">
         <is>
-          <t>2026-09-07T09:41:00+00:00</t>
+          <t>2026-09-16T07:59:00+00:00</t>
         </is>
       </c>
       <c r="K489" s="9" t="inlineStr">
@@ -56782,18 +56752,18 @@
       </c>
       <c r="L489" s="9" t="inlineStr">
         <is>
-          <t>EP-MN23-260905-57</t>
+          <t>EP-GU09-260913-17</t>
         </is>
       </c>
       <c r="M489" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05T19:17:00+00:00</t>
+          <t>2026-09-13T22:23:00+00:00</t>
         </is>
       </c>
       <c r="N489" s="9" t="inlineStr"/>
       <c r="O489" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05T19:17:00+00:00</t>
+          <t>2026-09-13T22:23:00+00:00</t>
         </is>
       </c>
     </row>
@@ -56887,7 +56857,7 @@
     <row r="494">
       <c r="A494" s="9" t="inlineStr">
         <is>
-          <t>EP-ZA06-260901-47</t>
+          <t>EP-ZA06-260901-71</t>
         </is>
       </c>
       <c r="B494" s="9" t="inlineStr">
@@ -56915,7 +56885,7 @@
     <row r="495">
       <c r="A495" s="9" t="inlineStr">
         <is>
-          <t>EP-ZA04-260826-46</t>
+          <t>EP-ZA04-260826-70</t>
         </is>
       </c>
       <c r="B495" s="9" t="inlineStr">
@@ -56971,7 +56941,7 @@
     <row r="497">
       <c r="A497" s="9" t="inlineStr">
         <is>
-          <t>EP-ZA01-260705-44</t>
+          <t>EP-ZA01-260705-68</t>
         </is>
       </c>
       <c r="B497" s="9" t="inlineStr">
@@ -57161,7 +57131,7 @@
     <row r="502">
       <c r="A502" s="9" t="inlineStr">
         <is>
-          <t>cierre-EV-2011-0909--oper-2026-09-10T07:00:00.000Z</t>
+          <t>cierre-EV-2011-0809--oper-2026-08-10T04:19:00.000Z</t>
         </is>
       </c>
       <c r="B502" s="9" t="inlineStr">
@@ -57176,7 +57146,7 @@
       </c>
       <c r="D502" s="9" t="inlineStr">
         <is>
-          <t>{"hora": "01:59", "campo": "La Ceiba", "equipo": "P-201B"}</t>
+          <t>{"hora": "23:18", "campo": "La Ceiba", "equipo": "P-201B"}</t>
         </is>
       </c>
       <c r="E502" s="9" t="inlineStr">
@@ -57201,19 +57171,19 @@
       </c>
       <c r="I502" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T07:00:00+00:00</t>
+          <t>2026-08-10T04:19:00+00:00</t>
         </is>
       </c>
       <c r="J502" s="9" t="inlineStr">
         <is>
-          <t>TRIM · Por P-201B parado se empezaron a cerrar pozos de La Ceiba a las 01:59.</t>
+          <t>TRIM · Por P-201B parado se empezaron a cerrar pozos de La Ceiba a las 23:18.</t>
         </is>
       </c>
       <c r="K502" s="9" t="inlineStr"/>
       <c r="L502" s="9" t="inlineStr"/>
       <c r="M502" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EV-2011-0809</t>
         </is>
       </c>
       <c r="N502" s="9" t="inlineStr"/>
@@ -57287,7 +57257,7 @@
     <row r="504">
       <c r="A504" s="9" t="inlineStr">
         <is>
-          <t>parada-EP-LC01-251227-38--oper-2025-12-27T18:14:00.000Z</t>
+          <t>parada-EP-LC01-251227-54--oper-2025-12-27T18:14:00.000Z</t>
         </is>
       </c>
       <c r="B504" s="9" t="inlineStr">
@@ -57339,7 +57309,7 @@
       <c r="L504" s="9" t="inlineStr"/>
       <c r="M504" s="9" t="inlineStr">
         <is>
-          <t>EP-LC01-251227-38</t>
+          <t>EP-LC01-251227-54</t>
         </is>
       </c>
       <c r="N504" s="9" t="inlineStr"/>
@@ -57350,7 +57320,7 @@
     <row r="505">
       <c r="A505" s="9" t="inlineStr">
         <is>
-          <t>parte-PR-EP-GU09-260913-93--conf-2026-09-10T22:23:00.000Z</t>
+          <t>parte-PR-EP-GU09-260913-17--conf-2026-09-07T22:23:00.000Z</t>
         </is>
       </c>
       <c r="B505" s="9" t="inlineStr">
@@ -57365,7 +57335,7 @@
       </c>
       <c r="D505" s="9" t="inlineStr">
         <is>
-          <t>{"campo": "Guacamayo", "desde": "12 de sept, 12:35", "hasta": "14 de sept, 22:11", "parte": "aislamiento del motor y del cable", "accion": "Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.", "equipo": "GU-09"}</t>
+          <t>{"campo": "Guacamayo", "desde": "11 de sept, 07:47", "hasta": "16 de sept, 02:59", "parte": "aislamiento del motor y del cable", "accion": "Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.", "equipo": "GU-09"}</t>
         </is>
       </c>
       <c r="E505" s="9" t="inlineStr">
@@ -57390,12 +57360,12 @@
       </c>
       <c r="I505" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T22:23:00+00:00</t>
+          <t>2026-09-07T22:23:00+00:00</t>
         </is>
       </c>
       <c r="J505" s="9" t="inlineStr">
         <is>
-          <t>TRIM · GU-09 de Guacamayo: el vigía anticipa falla en aislamiento del motor y del cable; cruzaría su límite entre el 12 de sept, 12:35 y el 14 de sept, 22:11. Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.</t>
+          <t>TRIM · GU-09 de Guacamayo: el vigía anticipa falla en aislamiento del motor y del cable; cruzaría su límite entre el 11 de sept, 07:47 y el 16 de sept, 02:59. Programar la prueba de aislamiento desde superficie y tener listo el equipo de reemplazo y el taladro.</t>
         </is>
       </c>
       <c r="K505" s="9" t="inlineStr"/>
@@ -57403,7 +57373,7 @@
       <c r="M505" s="9" t="inlineStr"/>
       <c r="N505" s="9" t="inlineStr">
         <is>
-          <t>PR-EP-GU09-260913-93</t>
+          <t>PR-EP-GU09-260913-17</t>
         </is>
       </c>
       <c r="O505" s="9" t="inlineStr"/>
@@ -57491,10 +57461,10 @@
         </is>
       </c>
       <c r="C509" s="9" t="n">
-        <v>324688</v>
+        <v>338662</v>
       </c>
       <c r="D509" s="9" t="n">
-        <v>335098.0972222224</v>
+        <v>349521.5180555556</v>
       </c>
       <c r="E509" s="9" t="n">
         <v>30</v>
@@ -57503,7 +57473,7 @@
         <v>0</v>
       </c>
       <c r="G509" s="9" t="n">
-        <v>0.9689341798460919</v>
+        <v>0.9689303304815998</v>
       </c>
       <c r="H509" s="9" t="n">
         <v>0.15</v>
@@ -57519,7 +57489,7 @@
       </c>
       <c r="L509" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -57535,10 +57505,10 @@
         </is>
       </c>
       <c r="C510" s="9" t="n">
-        <v>180748</v>
+        <v>200031</v>
       </c>
       <c r="D510" s="9" t="n">
-        <v>179444.9708333333</v>
+        <v>198590.6708333334</v>
       </c>
       <c r="E510" s="9" t="n">
         <v>30</v>
@@ -57547,7 +57517,7 @@
         <v>0</v>
       </c>
       <c r="G510" s="9" t="n">
-        <v>1.007261441547319</v>
+        <v>1.007252753417986</v>
       </c>
       <c r="H510" s="9" t="n">
         <v>0.05000000000000004</v>
@@ -57563,7 +57533,7 @@
       </c>
       <c r="L510" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -57579,10 +57549,10 @@
         </is>
       </c>
       <c r="C511" s="9" t="n">
-        <v>466040</v>
+        <v>504058</v>
       </c>
       <c r="D511" s="9" t="n">
-        <v>485095.2208333333</v>
+        <v>524672.0541666667</v>
       </c>
       <c r="E511" s="9" t="n">
         <v>30</v>
@@ -57591,7 +57561,7 @@
         <v>0</v>
       </c>
       <c r="G511" s="9" t="n">
-        <v>0.9607185970610083</v>
+        <v>0.9607105924492055</v>
       </c>
       <c r="H511" s="9" t="n">
         <v>0.15</v>
@@ -57607,7 +57577,7 @@
       </c>
       <c r="L511" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -57651,7 +57621,7 @@
       </c>
       <c r="L512" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -57695,7 +57665,7 @@
       </c>
       <c r="L513" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -57905,28 +57875,28 @@
         </is>
       </c>
       <c r="C517" s="9" t="n">
-        <v>324688</v>
+        <v>338662</v>
       </c>
       <c r="D517" s="9" t="n">
-        <v>346379.4352822801</v>
+        <v>346378.0591922146</v>
       </c>
       <c r="E517" s="9" t="n">
-        <v>21691.43528228009</v>
+        <v>7716.059192214569</v>
       </c>
       <c r="F517" s="9" t="n">
-        <v>21691.43528228031</v>
+        <v>7716.059192214809</v>
       </c>
       <c r="G517" s="9" t="n">
-        <v>-2.219167072325945e-10</v>
+        <v>-2.401066012680531e-10</v>
       </c>
       <c r="H517" s="9" t="n">
-        <v>3253.715293317683</v>
+        <v>1157.40887996932</v>
       </c>
       <c r="I517" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J517" s="9" t="n">
-        <v>21691.43528228031</v>
+        <v>7716.059192214809</v>
       </c>
       <c r="K517" s="9" t="n">
         <v>0</v>
@@ -57938,13 +57908,13 @@
         <v>0</v>
       </c>
       <c r="N517" s="9" t="n">
-        <v>21691.43528228031</v>
+        <v>7716.059192214809</v>
       </c>
       <c r="O517" s="9" t="n">
-        <v>21493.77069097883</v>
+        <v>7476.615648635969</v>
       </c>
       <c r="P517" s="9" t="n">
-        <v>21493.77069097883</v>
+        <v>7476.615648635969</v>
       </c>
       <c r="Q517" s="9" t="n">
         <v>0</v>
@@ -57953,10 +57923,10 @@
         <v>0</v>
       </c>
       <c r="S517" s="9" t="n">
-        <v>0</v>
+        <v>54.99592875553537</v>
       </c>
       <c r="T517" s="9" t="n">
-        <v>93.73766653767919</v>
+        <v>97.77235913550382</v>
       </c>
       <c r="U517" s="9" t="n">
         <v>327000</v>
@@ -57968,7 +57938,7 @@
         <v>0</v>
       </c>
       <c r="X517" s="9" t="n">
-        <v>1041188.893549445</v>
+        <v>370370.8412263042</v>
       </c>
       <c r="Y517" s="9" t="b">
         <v>0</v>
@@ -57991,17 +57961,17 @@
       </c>
       <c r="AD517" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl": 20738.85724968679, "tipo": "reinyeccion"}, {"bbl": 754.9134412920458, "tipo": "electrosumergible"}, {"bbl": 197.66459130147743, "tipo": "energia"}]</t>
+          <t>[{"bbl": 6436.065217892938, "tipo": "electrosumergible"}, {"bbl": 1040.5504307430315, "tipo": "reinyeccion"}, {"bbl": 239.44354357884006, "tipo": "energia"}]</t>
         </is>
       </c>
       <c r="AE517" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl":20738.85724968679,"tipo":"reinyeccion","pozos":18,"equipo":"P-201B","partes":[{"bbl":14649.470625413454,"parte":"sello"},{"bbl":6089.386624273328,"parte":"rodamientos"}],"campoId":"ceiba","eventos":2,"tolerancia":3110.8285881692505},{"bbl":216.65435548454434,"tipo":"electrosumergible","pozos":1,"equipo":"LC-16","partes":[{"bbl":216.65435548454434,"parte":"admision"}],"campoId":"ceiba","eventos":2,"tolerancia":32.498159689858475},{"bbl":197.66459130147743,"tipo":"energia","pozos":2,"equipo":"SE-2","partes":[],"campoId":"ceiba","eventos":2,"tolerancia":29.649692535436152},{"bbl":136.11372039771268,"tipo":"electrosumergible","pozos":1,"equipo":"LC-11","partes":[{"bbl":136.11372039771268,"parte":"bomba"}],"campoId":"ceiba","eventos":1,"tolerancia":20.41706519134548},{"bbl":131.4016050772528,"tipo":"electrosumergible","pozos":1,"equipo":"LC-07","partes":[{"bbl":131.4016050772528,"parte":"motor"}],"campoId":"ceiba","eventos":1,"tolerancia":19.71024516785824},{"bbl":94.61103969430506,"tipo":"electrosumergible","pozos":1,"equipo":"LC-14","partes":[{"bbl":66.61960783208463,"parte":"bomba"},{"bbl":27.991431862220434,"parte":"admision"}],"campoId":"ceiba","eventos":2,"tolerancia":14.191668223012627},{"bbl":60.830226107504224,"tipo":"electrosumergible","pozos":1,"equipo":"LC-08","partes":[{"bbl":60.830226107504224,"parte":"admision"}],"campoId":"ceiba","eventos":1,"tolerancia":9.124545888544908},{"bbl":54.85378625653688,"tipo":"electrosumergible","pozos":1,"equipo":"LC-09","parte… [recortado para el Excel: 2212 caracteres]</t>
+          <t>[{"bbl":3677.2278693078233,"tipo":"electrosumergible","pozos":1,"equipo":"LC-11","fallas":1,"partes":[{"bbl":3677.2278693078233,"parte":"aislamiento"}],"campoId":"ceiba","eventos":1,"disparos":0,"tolerancia":551.5841806601529},{"bbl":2125.5969683085755,"tipo":"electrosumergible","pozos":1,"equipo":"LC-04","fallas":1,"partes":[{"bbl":2125.5969683085755,"parte":"aislamiento"}],"campoId":"ceiba","eventos":1,"disparos":0,"tolerancia":318.839545538696},{"bbl":1040.5504307430315,"tipo":"reinyeccion","pozos":2,"equipo":"P-201B","fallas":1,"partes":[{"bbl":1040.5504307430315,"parte":"rodamientos"}],"campoId":"ceiba","eventos":1,"disparos":0,"tolerancia":156.0825658307318},{"bbl":239.44354357884006,"tipo":"energia","pozos":3,"equipo":"SE-2","partes":[],"campoId":"ceiba","eventos":3,"tolerancia":35.91653653227523},{"bbl":216.6534947639708,"tipo":"electrosumergible","pozos":1,"equipo":"LC-16","fallas":0,"partes":[{"bbl":216.6534947639708,"parte":"admision"}],"campoId":"ceiba","eventos":2,"disparos":2,"tolerancia":32.498030581747145},{"bbl":131.4010830472911,"tipo":"electrosumergible","pozos":1,"equipo":"LC-07","fallas":0,"partes":[{"bbl":131.4010830472911,"parte":"motor"}],"campoId":"ceiba","eventos":1,"disparos":1,"tolerancia":19.71016686334648},{"bbl":94.61066382524777,"tipo":"electrosumergible","pozos":1,"equipo":"LC-14","fallas":0,"partes":[{"bbl":66.61934316689045,"parte":"bomba"},{"bbl":27.991320658357328,"parte":"admision"}],"campoId":"ceiba","eventos":2,"disparos":2,"tolerancia"… [recortado para el Excel: 2684 caracteres]</t>
         </is>
       </c>
       <c r="AF517" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl":14649.470625413454,"horas":34.76,"parte":"sello","fallas":1,"equipos":[{"bbl":14649.470625413454,"equipo":"P-201B","campoId":"ceiba"}],"familia":"inyeccion","disparos":0},{"bbl":6089.386624273328,"horas":15.991111111111111,"parte":"rodamientos","fallas":1,"equipos":[{"bbl":6089.386624273328,"equipo":"P-201B","campoId":"ceiba"}],"familia":"inyeccion","disparos":0},{"bbl":395.9845589162674,"horas":12.699999999999998,"parte":"admision","fallas":0,"equipos":[{"bbl":216.65435548454434,"equipo":"LC-16","campoId":"ceiba"},{"bbl":60.830226107504224,"equipo":"LC-08","campoId":"ceiba"},{"bbl":54.85378625653688,"equipo":"LC-09","campoId":"ceiba"},{"bbl":27.991431862220434,"equipo":"LC-14","campoId":"ceiba"},{"bbl":19.93380213745866,"equipo":"LC-02","campoId":"ceiba"},{"bbl":15.720957068002841,"equipo":"LC-12","campoId":"ceiba"}],"familia":"electrosumergible","disparos":7},{"bbl":202.7333282297973,"horas":5.116666666666667,"parte":"bomba","fallas":0,"equipos":[{"bbl":136.11372039771268,"equipo":"LC-11","campoId":"ceiba"},{"bbl":66.61960783208463,"equipo":"LC-14","campoId":"ceiba"}],"familia":"electrosumergible","disparos":2},{"bbl":131.4016050772528,"horas":3.9166666666666665,"parte":"motor","fallas":0,"equipos":[{"bbl":131.4016050772528,"equipo":"LC-07","campoId":"ceiba"}],"familia":"electrosumergible","disparos":1},{"bbl":24.793949068728327,"horas":1.6333333333333333,"parte":"aislamiento","fallas":0,"equipos":[{"bbl":24.793949068728327,"equipo":"LC-01","campoId":"ceiba"}],"fami… [recortado para el Excel: 1539 caracteres]</t>
+          <t>[{"bbl": 5842.061805922908, "horas": 148.31666666666666, "parte": "aislamiento", "fallas": 2, "equipos": [{"bbl": 3677.2278693078233, "equipo": "LC-11", "campoId": "ceiba"}, {"bbl": 2125.5969683085755, "equipo": "LC-04", "campoId": "ceiba"}, {"bbl": 24.793850567768047, "equipo": "LC-01", "campoId": "ceiba"}, {"bbl": 14.443117738741348, "equipo": "LC-12", "campoId": "ceiba"}], "familia": "electrosumergible", "disparos": 2}, {"bbl": 1040.5504307430315, "horas": 15.991111111111111, "parte": "rodamientos", "fallas": 1, "equipos": [{"bbl": 1040.5504307430315, "equipo": "P-201B", "campoId": "ceiba"}], "familia": "inyeccion", "disparos": 0}, {"bbl": 395.9829857558483, "horas": 12.699999999999998, "parte": "admision", "fallas": 0, "equipos": [{"bbl": 216.6534947639708, "equipo": "LC-16", "campoId": "ceiba"}, {"bbl": 60.829984442262884, "equipo": "LC-08", "campoId": "ceiba"}, {"bbl": 54.85356833438957, "equipo": "LC-09", "campoId": "ceiba"}, {"bbl": 27.991320658357328, "equipo": "LC-14", "campoId": "ceiba"}, {"bbl": 19.933722944803744, "equipo": "LC-02", "campoId": "ceiba"}, {"bbl": 15.720894612063956, "equipo": "LC-12", "campoId": "ceiba"}], "familia": "electrosumergible", "disparos": 7}, {"bbl": 131.4010830472911, "horas": 3.9166666666666665, "parte": "motor", "fallas": 0, "equipos": [{"bbl": 131.4010830472911, "equipo": "LC-07", "campoId": "ceiba"}], "familia": "electrosumergible", "disparos": 1}, {"bbl": 66.61934316689045, "horas": 1.9833333333333334, "parte": "bomba", "fallas": 0, "equipos": [{"bbl": 66.61934316689045, "equipo": "LC-14", "campoId": "ceiba"}], "familia": "electrosumergible", "disparos": 1}]</t>
         </is>
       </c>
       <c r="AG517" s="9" t="inlineStr">
@@ -58010,11 +57980,11 @@
         </is>
       </c>
       <c r="AH517" s="9" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="AI517" s="9" t="inlineStr">
         <is>
-          <t>fa38baaa420730961c4855543e7a4d6d3f086e665341f9534f30d2c21bd205ac</t>
+          <t>9439920a3b191e5defc44bbf5a02780c01f4c477b4232259de355bd618234cb8</t>
         </is>
       </c>
       <c r="AJ517" s="9" t="n">
@@ -58022,7 +57992,7 @@
       </c>
       <c r="AK517" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -58038,28 +58008,28 @@
         </is>
       </c>
       <c r="C518" s="9" t="n">
-        <v>180748</v>
+        <v>200031</v>
       </c>
       <c r="D518" s="9" t="n">
-        <v>206429.1670921492</v>
+        <v>206427.3865382355</v>
       </c>
       <c r="E518" s="9" t="n">
-        <v>25681.1670921492</v>
+        <v>6396.386538235471</v>
       </c>
       <c r="F518" s="9" t="n">
-        <v>25681.16709214917</v>
+        <v>6396.386538235546</v>
       </c>
       <c r="G518" s="9" t="n">
-        <v>3.637978807091713e-11</v>
+        <v>-7.548806024715304e-11</v>
       </c>
       <c r="H518" s="9" t="n">
-        <v>1284.058355025105</v>
+        <v>319.8193285885733</v>
       </c>
       <c r="I518" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J518" s="9" t="n">
-        <v>25681.16709214917</v>
+        <v>6396.386538235546</v>
       </c>
       <c r="K518" s="9" t="n">
         <v>0</v>
@@ -58071,13 +58041,13 @@
         <v>0</v>
       </c>
       <c r="N518" s="9" t="n">
-        <v>25681.16709214917</v>
+        <v>6396.386538235546</v>
       </c>
       <c r="O518" s="9" t="n">
-        <v>25681.16709214917</v>
+        <v>6396.386538235546</v>
       </c>
       <c r="P518" s="9" t="n">
-        <v>25681.16709214917</v>
+        <v>6396.386538235546</v>
       </c>
       <c r="Q518" s="9" t="n">
         <v>0</v>
@@ -58089,7 +58059,7 @@
         <v>0</v>
       </c>
       <c r="T518" s="9" t="n">
-        <v>87.55933211672301</v>
+        <v>96.90138665924994</v>
       </c>
       <c r="U518" s="9" t="n">
         <v>189000</v>
@@ -58101,7 +58071,7 @@
         <v>0</v>
       </c>
       <c r="X518" s="9" t="n">
-        <v>1232696.02042316</v>
+        <v>307026.5538353045</v>
       </c>
       <c r="Y518" s="9" t="b">
         <v>0</v>
@@ -58124,17 +58094,17 @@
       </c>
       <c r="AD518" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl": 25681.167092149168, "tipo": "electrosumergible"}]</t>
+          <t>[{"bbl": 6396.386538235546, "tipo": "electrosumergible"}]</t>
         </is>
       </c>
       <c r="AE518" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl":11765.572580789412,"tipo":"electrosumergible","pozos":1,"equipo":"GU-05","partes":[{"bbl":11765.572580789412,"parte":"bomba"}],"campoId":"guacamayo","eventos":1,"tolerancia":588.2786290938159},{"bbl":10510.289097464643,"tipo":"electrosumergible","pozos":1,"equipo":"GU-09","partes":[{"bbl":10510.289097464643,"parte":"aislamiento"}],"campoId":"guacamayo","eventos":1,"tolerancia":525.5144549675836},{"bbl":3004.389479136126,"tipo":"electrosumergible","pozos":1,"equipo":"GU-07","partes":[{"bbl":3004.389479136126,"parte":"aislamiento"}],"campoId":"guacamayo","eventos":1,"tolerancia":150.21947429016225},{"bbl":146.71602280671328,"tipo":"electrosumergible","pozos":1,"equipo":"GU-06","partes":[{"bbl":146.71602280671328,"parte":"admision"}],"campoId":"guacamayo","eventos":2,"tolerancia":7.335818324685073},{"bbl":73.68117444918641,"tipo":"electrosumergible","pozos":1,"equipo":"GU-01","partes":[{"bbl":73.68117444918641,"parte":"admision"}],"campoId":"guacamayo","eventos":1,"tolerancia":3.6840845059328466},{"bbl":61.37090076183136,"tipo":"electrosumergible","pozos":1,"equipo":"GU-12","partes":[{"bbl":61.37090076183136,"parte":"admision"}],"campoId":"guacamayo","eventos":1,"tolerancia":3.0685520188876407},{"bbl":43.3038481411885,"tipo":"electrosumergible","pozos":1,"equipo":"GU-03","partes":[{"bbl":43.3038481411885,"parte":"admision"}],"campoId":"guacamayo","eventos":1,"tolerancia":2.1652265021614623},{"bbl":34.04963364697251,"tipo":"electrosumergible","pozos":1,"equipo":"GU-10","p… [recortado para el Excel: 2019 caracteres]</t>
+          <t>[{"bbl":2393.7361684978446,"tipo":"electrosumergible","pozos":1,"equipo":"GU-05","fallas":1,"partes":[{"bbl":2393.7361684978446,"parte":"bomba"}],"campoId":"guacamayo","eventos":1,"disparos":0,"tolerancia":119.68680869200017},{"bbl":2054.974684128855,"tipo":"electrosumergible","pozos":1,"equipo":"GU-09","fallas":1,"partes":[{"bbl":2054.974684128855,"parte":"aislamiento"}],"campoId":"guacamayo","eventos":1,"disparos":0,"tolerancia":102.74873468899787},{"bbl":1546.763208948574,"tipo":"electrosumergible","pozos":1,"equipo":"GU-07","fallas":1,"partes":[{"bbl":1546.763208948574,"parte":"aislamiento"}],"campoId":"guacamayo","eventos":1,"disparos":0,"tolerancia":77.33816109491865},{"bbl":146.71475730827487,"tipo":"electrosumergible","pozos":1,"equipo":"GU-06","fallas":0,"partes":[{"bbl":146.71475730827487,"parte":"admision"}],"campoId":"guacamayo","eventos":2,"disparos":2,"tolerancia":7.33575504961493},{"bbl":73.6805389125257,"tipo":"electrosumergible","pozos":1,"equipo":"GU-01","fallas":0,"partes":[{"bbl":73.6805389125257,"parte":"admision"}],"campoId":"guacamayo","eventos":1,"disparos":1,"tolerancia":3.6840527288774156},{"bbl":61.370371407384624,"tipo":"electrosumergible","pozos":1,"equipo":"GU-12","fallas":0,"partes":[{"bbl":61.370371407384624,"parte":"admision"}],"campoId":"guacamayo","eventos":1,"disparos":1,"tolerancia":3.068525551105091},{"bbl":43.30347462402825,"tipo":"electrosumergible","pozos":1,"equipo":"GU-03","fallas":0,"partes":[{"bbl":43.30347462402825,"parte":"admisi… [recortado para el Excel: 2265 caracteres]</t>
         </is>
       </c>
       <c r="AF518" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl": 13514.678576600769, "horas": 532.55, "parte": "aislamiento", "fallas": 2, "equipos": [{"bbl": 10510.289097464643, "equipo": "GU-09", "campoId": "guacamayo"}, {"bbl": 3004.389479136126, "equipo": "GU-07", "campoId": "guacamayo"}], "familia": "electrosumergible", "disparos": 0}, {"bbl": 11784.032045679991, "horas": 578.9833333333333, "parte": "bomba", "fallas": 1, "equipos": [{"bbl": 11765.572580789412, "equipo": "GU-05", "campoId": "guacamayo"}, {"bbl": 18.459464890579, "equipo": "GU-11", "campoId": "guacamayo"}], "familia": "electrosumergible", "disparos": 1}, {"bbl": 382.45646986840495, "horas": 15.533333333333333, "parte": "admision", "fallas": 0, "equipos": [{"bbl": 146.71602280671328, "equipo": "GU-06", "campoId": "guacamayo"}, {"bbl": 73.68117444918641, "equipo": "GU-01", "campoId": "guacamayo"}, {"bbl": 61.37090076183136, "equipo": "GU-12", "campoId": "guacamayo"}, {"bbl": 43.3038481411885, "equipo": "GU-03", "campoId": "guacamayo"}, {"bbl": 34.04963364697251, "equipo": "GU-10", "campoId": "guacamayo"}, {"bbl": 23.334890062512898, "equipo": "GU-08", "campoId": "guacamayo"}], "familia": "electrosumergible", "disparos": 7}]</t>
+          <t>[{"bbl": 3601.7378930774294, "horas": 141.78333333333333, "parte": "aislamiento", "fallas": 2, "equipos": [{"bbl": 2054.974684128855, "equipo": "GU-09", "campoId": "guacamayo"}, {"bbl": 1546.763208948574, "equipo": "GU-07", "campoId": "guacamayo"}], "familia": "electrosumergible", "disparos": 0}, {"bbl": 2412.1954741663867, "horas": 118.56666666666666, "parte": "bomba", "fallas": 1, "equipos": [{"bbl": 2393.7361684978446, "equipo": "GU-05", "campoId": "guacamayo"}, {"bbl": 18.45930566854212, "equipo": "GU-11", "campoId": "guacamayo"}], "familia": "electrosumergible", "disparos": 1}, {"bbl": 382.45317099173064, "horas": 15.533333333333333, "parte": "admision", "fallas": 0, "equipos": [{"bbl": 146.71475730827487, "equipo": "GU-06", "campoId": "guacamayo"}, {"bbl": 73.6805389125257, "equipo": "GU-01", "campoId": "guacamayo"}, {"bbl": 61.370371407384624, "equipo": "GU-12", "campoId": "guacamayo"}, {"bbl": 43.30347462402825, "equipo": "GU-03", "campoId": "guacamayo"}, {"bbl": 34.049339952000516, "equipo": "GU-10", "campoId": "guacamayo"}, {"bbl": 23.334688787516683, "equipo": "GU-08", "campoId": "guacamayo"}], "familia": "electrosumergible", "disparos": 7}]</t>
         </is>
       </c>
       <c r="AG518" s="9" t="inlineStr">
@@ -58147,7 +58117,7 @@
       </c>
       <c r="AI518" s="9" t="inlineStr">
         <is>
-          <t>30dd89011fc9f3e48856548e50adbc9ed6a9b9b6d51b21a2bd651d4d900d6013</t>
+          <t>ed542826fa682035e79cb219d14b4c54a27cc7c262f0b887d70ae3512459e800</t>
         </is>
       </c>
       <c r="AJ518" s="9" t="n">
@@ -58155,7 +58125,7 @@
       </c>
       <c r="AK518" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -58171,58 +58141,58 @@
         </is>
       </c>
       <c r="C519" s="9" t="n">
-        <v>466040</v>
+        <v>504058</v>
       </c>
       <c r="D519" s="9" t="n">
-        <v>519601.7710646552</v>
+        <v>519597.4417943752</v>
       </c>
       <c r="E519" s="9" t="n">
-        <v>53561.77106465516</v>
+        <v>15539.44179437525</v>
       </c>
       <c r="F519" s="9" t="n">
-        <v>53561.77106465516</v>
+        <v>15539.44179437547</v>
       </c>
       <c r="G519" s="9" t="n">
-        <v>-7.275957614183426e-12</v>
+        <v>-2.237356966361403e-10</v>
       </c>
       <c r="H519" s="9" t="n">
-        <v>8034.265659817542</v>
+        <v>2330.916269532946</v>
       </c>
       <c r="I519" s="9" t="n">
         <v>0</v>
       </c>
       <c r="J519" s="9" t="n">
-        <v>53455.27807683372</v>
+        <v>15432.94969384301</v>
       </c>
       <c r="K519" s="9" t="n">
-        <v>106.4929878214432</v>
+        <v>106.4921005324599</v>
       </c>
       <c r="L519" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M519" s="9" t="n">
-        <v>0</v>
+        <v>1385.081813219098</v>
       </c>
       <c r="N519" s="9" t="n">
-        <v>53561.77106465516</v>
+        <v>14154.35998115637</v>
       </c>
       <c r="O519" s="9" t="n">
-        <v>50321.01571530234</v>
+        <v>10909.28708666452</v>
       </c>
       <c r="P519" s="9" t="n">
-        <v>40483.19390065684</v>
+        <v>7120.750217426161</v>
       </c>
       <c r="Q519" s="9" t="n">
         <v>0</v>
       </c>
       <c r="R519" s="9" t="n">
-        <v>9837.821814645504</v>
+        <v>3788.536869238364</v>
       </c>
       <c r="S519" s="9" t="n">
-        <v>4762.241668271593</v>
+        <v>200.6468983049642</v>
       </c>
       <c r="T519" s="9" t="n">
-        <v>89.69176510793872</v>
+        <v>97.00933058086055</v>
       </c>
       <c r="U519" s="9" t="n">
         <v>501000</v>
@@ -58234,7 +58204,7 @@
         <v>0</v>
       </c>
       <c r="X519" s="9" t="n">
-        <v>2570965.011103444</v>
+        <v>745893.2061300157</v>
       </c>
       <c r="Y519" s="9" t="b">
         <v>0</v>
@@ -58257,17 +58227,17 @@
       </c>
       <c r="AD519" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl": 40483.193900656835, "tipo": "electrosumergible"}, {"bbl": 9837.821814645504, "tipo": "reinyeccion"}, {"bbl": 3022.4513959757824, "tipo": "transporte"}, {"bbl": 111.81096555559127, "tipo": "energia"}, {"bbl": 106.49298782144315, "tipo": "declarada"}]</t>
+          <t>[{"bbl": 7120.750217426161, "tipo": "electrosumergible"}, {"bbl": 3788.5368692383636, "tipo": "reinyeccion"}, {"bbl": 3026.7707600016465, "tipo": "transporte"}, {"bbl": 1385.081813219098, "tipo": "programada"}, {"bbl": 111.81003395774638, "tipo": "energia"}, {"bbl": 106.49210053245986, "tipo": "declarada"}]</t>
         </is>
       </c>
       <c r="AE519" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl":18638.10090274974,"tipo":"electrosumergible","pozos":1,"equipo":"MN-41","partes":[{"bbl":18638.10090274974,"parte":"aislamiento"}],"campoId":"morichal","eventos":1,"tolerancia":2795.7151354341186},{"bbl":9837.821814645504,"tipo":"reinyeccion","pozos":8,"equipo":"P-201B","partes":[],"campoId":"morichal","eventos":1,"tolerancia":1475.6732723337602},{"bbl":8645.059653938104,"tipo":"electrosumergible","pozos":1,"equipo":"MN-16","partes":[{"bbl":8580.551403139612,"parte":"bomba"},{"bbl":64.50825079849228,"parte":"admision"}],"campoId":"morichal","eventos":2,"tolerancia":1296.7589481568727},{"bbl":7783.060897216348,"tipo":"electrosumergible","pozos":1,"equipo":"MN-05","partes":[{"bbl":7783.060897216348,"parte":"bomba"}],"campoId":"morichal","eventos":1,"tolerancia":1167.4591346081925},{"bbl":4944.974735845033,"tipo":"electrosumergible","pozos":1,"equipo":"MN-23","partes":[{"bbl":4944.974735845033,"parte":"admision"}],"campoId":"morichal","eventos":1,"tolerancia":741.7462103897301},{"bbl":3022.4513959757824,"tipo":"transporte","pozos":3,"equipo":"MPP-301","partes":[{"bbl":3022.4513959757824,"parte":"sello"}],"campoId":"morichal","eventos":1,"tolerancia":453.3677096452056},{"bbl":111.81096555559127,"tipo":"energia","pozos":5,"equipo":"SE-2","partes":[],"campoId":"morichal","eventos":5,"tolerancia":16.771650672788528},{"bbl":106.49298782144315,"tipo":"declarada","pozos":1,"equipo":"MN-22","partes":[],"campoId":"morichal","eventos":1,"tolerancia":15.973949105207163},{"bbl":86.2… [recortado para el Excel: 3776 caracteres]</t>
+          <t>[{"bbl":3831.687452362273,"tipo":"electrosumergible","pozos":1,"equipo":"MN-41","fallas":1,"partes":[{"bbl":3831.687452362273,"parte":"aislamiento"}],"campoId":"morichal","eventos":1,"disparos":0,"tolerancia":574.7531179588469},{"bbl":3788.5368692383636,"tipo":"reinyeccion","pozos":2,"equipo":"P-201B","fallas":1,"partes":[],"campoId":"morichal","eventos":1,"disparos":0,"tolerancia":568.2805305345369},{"bbl":3026.7707600016465,"tipo":"transporte","pozos":3,"equipo":"MPP-301","fallas":1,"partes":[{"bbl":3026.7707600016465,"parte":"sello"}],"campoId":"morichal","eventos":1,"disparos":0,"tolerancia":454.01561424873296},{"bbl":1958.1256668110398,"tipo":"electrosumergible","pozos":1,"equipo":"MN-33","fallas":1,"partes":[{"bbl":1958.1256668110398,"parte":"aislamiento"}],"campoId":"morichal","eventos":1,"disparos":0,"tolerancia":293.71885011703205},{"bbl":794.4356066610593,"tipo":"electrosumergible","pozos":1,"equipo":"MN-23","fallas":1,"partes":[{"bbl":794.4356066610593,"parte":"admision"}],"campoId":"morichal","eventos":2,"disparos":1,"tolerancia":119.16534116068624},{"bbl":743.7074187392067,"tipo":"programada","pozos":1,"equipo":"MN-16","partes":[],"campoId":"morichal","eventos":1,"tolerancia":111.55611319930645},{"bbl":641.3743944798914,"tipo":"programada","pozos":1,"equipo":"MN-05","partes":[],"campoId":"morichal","eventos":1,"tolerancia":96.20615948433881},{"bbl":111.81003395774638,"tipo":"energia","pozos":5,"equipo":"SE-2","partes":[],"campoId":"morichal","eventos":5,"toleranc… [recortado para el Excel: 4452 caracteres]</t>
         </is>
       </c>
       <c r="AF519" s="9" t="inlineStr">
         <is>
-          <t>[{"bbl":18755.5967871703,"horas":673.8666666666667,"parte":"aislamiento","fallas":1,"equipos":[{"bbl":18638.10090274974,"equipo":"MN-41","campoId":"morichal"},{"bbl":40.3982170064154,"equipo":"MN-27","campoId":"morichal"},{"bbl":38.71896095863584,"equipo":"MN-12","campoId":"morichal"},{"bbl":38.37870645551007,"equipo":"MN-13","campoId":"morichal"}],"familia":"electrosumergible","disparos":3},{"bbl":16585.316797267173,"horas":770.8,"parte":"bomba","fallas":2,"equipos":[{"bbl":8580.551403139612,"equipo":"MN-16","campoId":"morichal"},{"bbl":7783.060897216348,"equipo":"MN-05","campoId":"morichal"},{"bbl":76.24035949940743,"equipo":"MN-19","campoId":"morichal"},{"bbl":52.08162261178511,"equipo":"MN-24","campoId":"morichal"},{"bbl":35.04487949056989,"equipo":"MN-01","campoId":"morichal"},{"bbl":33.75858403561598,"equipo":"MN-37","campoId":"morichal"},{"bbl":24.57905127383653,"equipo":"MN-20","campoId":"morichal"}],"familia":"electrosumergible","disparos":5},{"bbl":5115.716447010624,"horas":451.5,"parte":"admision","fallas":1,"equipos":[{"bbl":4944.974735845033,"equipo":"MN-23","campoId":"morichal"},{"bbl":64.50825079849228,"equipo":"MN-16","campoId":"morichal"},{"bbl":60.94024867551848,"equipo":"MN-17","campoId":"morichal"},{"bbl":23.466886064599933,"equipo":"MN-11","campoId":"morichal"},{"bbl":11.806164092771946,"equipo":"MN-18","campoId":"morichal"},{"bbl":10.020161534207835,"equipo":"MN-19","campoId":"morichal"}],"familia":"electrosumergible","disparos":5},{"bbl":3022.4513959757… [recortado para el Excel: 1860 caracteres]</t>
+          <t>[{"bbl":5907.3080246298505,"horas":248.63333333333335,"parte":"aislamiento","fallas":2,"equipos":[{"bbl":3831.687452362273,"equipo":"MN-41","campoId":"morichal"},{"bbl":1958.1256668110398,"equipo":"MN-33","campoId":"morichal"},{"bbl":40.39788041248909,"equipo":"MN-27","campoId":"morichal"},{"bbl":38.71863835610392,"equipo":"MN-12","campoId":"morichal"},{"bbl":38.37838668794483,"equipo":"MN-13","campoId":"morichal"}],"familia":"electrosumergible","disparos":3},{"bbl":3026.7707600016465,"horas":45.40277777777778,"parte":"sello","fallas":1,"equipos":[{"bbl":3026.7707600016465,"equipo":"MPP-301","campoId":"morichal"}],"familia":"multifasica","disparos":0},{"bbl":965.1758952236935,"horas":79.86666666666669,"parte":"admision","fallas":1,"equipos":[{"bbl":794.4356066610593,"equipo":"MN-23","campoId":"morichal"},{"bbl":64.50771332216229,"equipo":"MN-16","campoId":"morichal"},{"bbl":60.939740927427316,"equipo":"MN-17","campoId":"morichal"},{"bbl":23.466690540839135,"equipo":"MN-11","campoId":"morichal"},{"bbl":11.806065724986903,"equipo":"MN-18","campoId":"morichal"},{"bbl":10.020078047218485,"equipo":"MN-19","campoId":"morichal"}],"familia":"electrosumergible","disparos":6},{"bbl":221.70264969139626,"horas":14.333333333333332,"parte":"bomba","fallas":0,"equipos":[{"bbl":76.23972427231456,"equipo":"MN-19","campoId":"morichal"},{"bbl":52.08118867288526,"equipo":"MN-24","campoId":"morichal"},{"bbl":35.044587500119356,"equipo":"MN-01","campoId":"morichal"},{"bbl":33.75830276245125,"equip… [recortado para el Excel: 1829 caracteres]</t>
         </is>
       </c>
       <c r="AG519" s="9" t="inlineStr">
@@ -58276,11 +58246,11 @@
         </is>
       </c>
       <c r="AH519" s="9" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="AI519" s="9" t="inlineStr">
         <is>
-          <t>1507ccacd9b9322188f1eaf7547e6cf62b5d0d3302deb9bcba0dbd248bc2c21a</t>
+          <t>190cb266ba2594a2c185be30cfd7e7bad4d7bce844013f88ff09f73007458480</t>
         </is>
       </c>
       <c r="AJ519" s="9" t="n">
@@ -58288,7 +58258,7 @@
       </c>
       <c r="AK519" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -58421,7 +58391,7 @@
       </c>
       <c r="AK520" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -58552,7 +58522,7 @@
       </c>
       <c r="AK521" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -58688,12 +58658,12 @@
     <row r="525">
       <c r="A525" s="9" t="inlineStr">
         <is>
-          <t>EP-LC11-260910-79</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="B525" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C525" s="9" t="inlineStr">
@@ -58713,28 +58683,28 @@
       </c>
       <c r="F525" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T07:03:00+00:00</t>
+          <t>2026-09-27T05:00:00+00:00</t>
         </is>
       </c>
       <c r="G525" s="9" t="inlineStr">
         <is>
-          <t>2026-09-11T05:00:00+00:00</t>
+          <t>2026-09-28T05:00:00+00:00</t>
         </is>
       </c>
       <c r="H525" s="9" t="n">
-        <v>21.95</v>
+        <v>24</v>
       </c>
       <c r="I525" s="9" t="n">
         <v>1</v>
       </c>
       <c r="J525" s="9" t="n">
-        <v>1097</v>
+        <v>1076</v>
       </c>
       <c r="K525" s="9" t="n">
-        <v>0.9689341798460919</v>
+        <v>0.9689303304815998</v>
       </c>
       <c r="L525" s="9" t="n">
-        <v>972.1296440267092</v>
+        <v>1042.569035598201</v>
       </c>
       <c r="M525" s="9" t="b">
         <v>0</v>
@@ -58750,22 +58720,22 @@
       </c>
       <c r="Q525" s="9" t="inlineStr">
         <is>
-          <t>reinyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="R525" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="S525" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="T525" s="9" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="U525" s="9" t="inlineStr">
@@ -58775,7 +58745,7 @@
       </c>
       <c r="V525" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="W525" s="9" t="n">
@@ -58783,19 +58753,19 @@
       </c>
       <c r="X525" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="9" t="inlineStr">
         <is>
-          <t>EP-LC08-260910-85</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="B526" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C526" s="9" t="inlineStr">
@@ -58810,33 +58780,33 @@
       </c>
       <c r="E526" s="9" t="inlineStr">
         <is>
-          <t>LC-08</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="F526" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T07:06:00+00:00</t>
+          <t>2026-09-28T05:00:00+00:00</t>
         </is>
       </c>
       <c r="G526" s="9" t="inlineStr">
         <is>
-          <t>2026-09-11T05:00:00+00:00</t>
+          <t>2026-09-29T05:00:00+00:00</t>
         </is>
       </c>
       <c r="H526" s="9" t="n">
-        <v>21.9</v>
+        <v>24</v>
       </c>
       <c r="I526" s="9" t="n">
         <v>1</v>
       </c>
       <c r="J526" s="9" t="n">
-        <v>942</v>
+        <v>1076</v>
       </c>
       <c r="K526" s="9" t="n">
-        <v>0.9689341798460919</v>
+        <v>0.9689303304815998</v>
       </c>
       <c r="L526" s="9" t="n">
-        <v>832.8715976412044</v>
+        <v>1042.569035598201</v>
       </c>
       <c r="M526" s="9" t="b">
         <v>0</v>
@@ -58852,22 +58822,22 @@
       </c>
       <c r="Q526" s="9" t="inlineStr">
         <is>
-          <t>reinyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="R526" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="S526" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="T526" s="9" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="U526" s="9" t="inlineStr">
@@ -58877,7 +58847,7 @@
       </c>
       <c r="V526" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="W526" s="9" t="n">
@@ -58885,19 +58855,19 @@
       </c>
       <c r="X526" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="9" t="inlineStr">
         <is>
-          <t>EP-LC16-260910-95</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="B527" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C527" s="9" t="inlineStr">
@@ -58912,33 +58882,33 @@
       </c>
       <c r="E527" s="9" t="inlineStr">
         <is>
-          <t>LC-16</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="F527" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T07:42:00+00:00</t>
+          <t>2026-09-26T05:00:00+00:00</t>
         </is>
       </c>
       <c r="G527" s="9" t="inlineStr">
         <is>
-          <t>2026-09-11T05:00:00+00:00</t>
+          <t>2026-09-27T05:00:00+00:00</t>
         </is>
       </c>
       <c r="H527" s="9" t="n">
-        <v>21.3</v>
+        <v>24</v>
       </c>
       <c r="I527" s="9" t="n">
         <v>1</v>
       </c>
       <c r="J527" s="9" t="n">
-        <v>907</v>
+        <v>1076</v>
       </c>
       <c r="K527" s="9" t="n">
-        <v>0.9689341798460919</v>
+        <v>0.9689303304815998</v>
       </c>
       <c r="L527" s="9" t="n">
-        <v>779.9556797443597</v>
+        <v>1042.569035598201</v>
       </c>
       <c r="M527" s="9" t="b">
         <v>0</v>
@@ -58954,22 +58924,22 @@
       </c>
       <c r="Q527" s="9" t="inlineStr">
         <is>
-          <t>reinyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="R527" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="S527" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="T527" s="9" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="U527" s="9" t="inlineStr">
@@ -58979,7 +58949,7 @@
       </c>
       <c r="V527" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="W527" s="9" t="n">
@@ -58987,19 +58957,19 @@
       </c>
       <c r="X527" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="9" t="inlineStr">
         <is>
-          <t>EP-LC05-260910-82</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
       <c r="B528" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C528" s="9" t="inlineStr">
@@ -59014,33 +58984,33 @@
       </c>
       <c r="E528" s="9" t="inlineStr">
         <is>
-          <t>LC-05</t>
+          <t>LC-04</t>
         </is>
       </c>
       <c r="F528" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T07:06:00+00:00</t>
+          <t>2026-09-27T05:00:00+00:00</t>
         </is>
       </c>
       <c r="G528" s="9" t="inlineStr">
         <is>
-          <t>2026-09-11T05:00:00+00:00</t>
+          <t>2026-09-28T05:00:00+00:00</t>
         </is>
       </c>
       <c r="H528" s="9" t="n">
-        <v>21.9</v>
+        <v>24</v>
       </c>
       <c r="I528" s="9" t="n">
         <v>1</v>
       </c>
       <c r="J528" s="9" t="n">
-        <v>843</v>
+        <v>861</v>
       </c>
       <c r="K528" s="9" t="n">
-        <v>0.9689341798460919</v>
+        <v>0.9689303304815998</v>
       </c>
       <c r="L528" s="9" t="n">
-        <v>745.340506169358</v>
+        <v>834.2490145446576</v>
       </c>
       <c r="M528" s="9" t="b">
         <v>0</v>
@@ -59056,22 +59026,22 @@
       </c>
       <c r="Q528" s="9" t="inlineStr">
         <is>
-          <t>reinyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="R528" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-04</t>
         </is>
       </c>
       <c r="S528" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="T528" s="9" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="U528" s="9" t="inlineStr">
@@ -59081,7 +59051,7 @@
       </c>
       <c r="V528" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
       <c r="W528" s="9" t="n">
@@ -59089,19 +59059,19 @@
       </c>
       <c r="X528" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="9" t="inlineStr">
         <is>
-          <t>EP-LC04-260910-88</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
       <c r="B529" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C529" s="9" t="inlineStr">
@@ -59121,16 +59091,16 @@
       </c>
       <c r="F529" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T07:37:00+00:00</t>
+          <t>2026-09-28T05:00:00+00:00</t>
         </is>
       </c>
       <c r="G529" s="9" t="inlineStr">
         <is>
-          <t>2026-09-11T05:00:00+00:00</t>
+          <t>2026-09-29T05:00:00+00:00</t>
         </is>
       </c>
       <c r="H529" s="9" t="n">
-        <v>21.38333333333333</v>
+        <v>24</v>
       </c>
       <c r="I529" s="9" t="n">
         <v>1</v>
@@ -59139,10 +59109,10 @@
         <v>861</v>
       </c>
       <c r="K529" s="9" t="n">
-        <v>0.9689341798460919</v>
+        <v>0.9689303304815998</v>
       </c>
       <c r="L529" s="9" t="n">
-        <v>743.2956513273078</v>
+        <v>834.2490145446576</v>
       </c>
       <c r="M529" s="9" t="b">
         <v>0</v>
@@ -59158,22 +59128,22 @@
       </c>
       <c r="Q529" s="9" t="inlineStr">
         <is>
-          <t>reinyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="R529" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-04</t>
         </is>
       </c>
       <c r="S529" s="9" t="inlineStr">
         <is>
-          <t>inyeccion</t>
+          <t>electrosumergible</t>
         </is>
       </c>
       <c r="T529" s="9" t="inlineStr">
         <is>
-          <t>sello</t>
+          <t>aislamiento</t>
         </is>
       </c>
       <c r="U529" s="9" t="inlineStr">
@@ -59183,7 +59153,7 @@
       </c>
       <c r="V529" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0909</t>
+          <t>EP-LC04-260926-75</t>
         </is>
       </c>
       <c r="W529" s="9" t="n">
@@ -59191,7 +59161,7 @@
       </c>
       <c r="X529" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -59261,20 +59231,20 @@
         </is>
       </c>
       <c r="D533" s="9" t="n">
-        <v>672.3833333333333</v>
+        <v>635.35</v>
       </c>
       <c r="E533" s="9" t="n">
-        <v>31765.53815207427</v>
+        <v>31765.41195450876</v>
       </c>
       <c r="F533" s="9" t="n">
-        <v>2106.207888892236</v>
+        <v>3677.227869307823</v>
       </c>
       <c r="G533" s="9" t="n">
-        <v>29659.33026318206</v>
+        <v>28088.18408520094</v>
       </c>
       <c r="H533" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -59295,20 +59265,20 @@
         </is>
       </c>
       <c r="D534" s="9" t="n">
-        <v>675.8</v>
+        <v>718.3833333333333</v>
       </c>
       <c r="E534" s="9" t="n">
-        <v>27256.11847907058</v>
+        <v>27256.01019644739</v>
       </c>
       <c r="F534" s="9" t="n">
-        <v>1675.357175533548</v>
+        <v>60.82998444226288</v>
       </c>
       <c r="G534" s="9" t="n">
-        <v>25580.76130353706</v>
+        <v>27195.18021200514</v>
       </c>
       <c r="H534" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -59329,20 +59299,20 @@
         </is>
       </c>
       <c r="D535" s="9" t="n">
-        <v>671.3</v>
+        <v>699.3333333333334</v>
       </c>
       <c r="E535" s="9" t="n">
-        <v>26475.15753011462</v>
+        <v>26475.05235007924</v>
       </c>
       <c r="F535" s="9" t="n">
-        <v>1783.278948523489</v>
+        <v>756.7615028375318</v>
       </c>
       <c r="G535" s="9" t="n">
-        <v>24691.87858159115</v>
+        <v>25718.29084724172</v>
       </c>
       <c r="H535" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -59359,24 +59329,24 @@
       </c>
       <c r="C536" s="9" t="inlineStr">
         <is>
-          <t>LC-04</t>
+          <t>LC-05</t>
         </is>
       </c>
       <c r="D536" s="9" t="n">
-        <v>673.85</v>
+        <v>720</v>
       </c>
       <c r="E536" s="9" t="n">
-        <v>25021.75626034547</v>
+        <v>24552.69457440375</v>
       </c>
       <c r="F536" s="9" t="n">
-        <v>1604.19770734631</v>
+        <v>0</v>
       </c>
       <c r="G536" s="9" t="n">
-        <v>23417.55855299918</v>
+        <v>24552.69457440377</v>
       </c>
       <c r="H536" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -59393,24 +59363,24 @@
       </c>
       <c r="C537" s="9" t="inlineStr">
         <is>
-          <t>LC-05</t>
+          <t>LC-14</t>
         </is>
       </c>
       <c r="D537" s="9" t="n">
-        <v>676.8666666666667</v>
+        <v>717.1833333333333</v>
       </c>
       <c r="E537" s="9" t="n">
-        <v>24552.79211729998</v>
+        <v>24111.8312740346</v>
       </c>
       <c r="F537" s="9" t="n">
-        <v>1470.410774722144</v>
+        <v>94.61066382524777</v>
       </c>
       <c r="G537" s="9" t="n">
-        <v>23082.38134257785</v>
+        <v>24017.22061020936</v>
       </c>
       <c r="H537" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
     </row>
@@ -59474,7 +59444,7 @@
       </c>
       <c r="D541" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
       <c r="E541" s="9" t="inlineStr">
@@ -59485,7 +59455,7 @@
       <c r="F541" s="9" t="inlineStr"/>
       <c r="G541" s="9" t="inlineStr">
         <is>
-          <t>0bdcbf1d9fa5fc6420f2410de1af37e9f84cb3384e58d68515450756cff5c411</t>
+          <t>5419eeb481140b47545569f04ef157c614b65495e455f923feaf3d04cbc7f108</t>
         </is>
       </c>
     </row>
@@ -59505,7 +59475,7 @@
       </c>
       <c r="D542" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
       <c r="E542" s="9" t="inlineStr">
@@ -59536,7 +59506,7 @@
       </c>
       <c r="D543" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
       <c r="E543" s="9" t="inlineStr">
@@ -59547,7 +59517,7 @@
       <c r="F543" s="9" t="inlineStr"/>
       <c r="G543" s="9" t="inlineStr">
         <is>
-          <t>680d5233961f9946f8b3167c52b76304462ab6b1b2f260421d83a2f7dcdc8bbb</t>
+          <t>3ee3116ec3bc84c4293321d097291669814f0af8cfa69fdeb7ff9233b5f63916</t>
         </is>
       </c>
     </row>
@@ -59567,7 +59537,7 @@
       </c>
       <c r="D544" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
       <c r="E544" s="9" t="inlineStr">
@@ -59578,7 +59548,7 @@
       <c r="F544" s="9" t="inlineStr"/>
       <c r="G544" s="9" t="inlineStr">
         <is>
-          <t>f71c87a7f8851963df606912d3ceca77669d2e5cf88a39e4c2e923255781655f</t>
+          <t>753d300b99414f01cc760a56987a7be0cb75f02cf6ed36bb72949f39b071cd8b</t>
         </is>
       </c>
     </row>
@@ -59598,7 +59568,7 @@
       </c>
       <c r="D545" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08T21:21:07.724868+00:00</t>
+          <t>2026-10-09T19:07:03.506705+00:00</t>
         </is>
       </c>
       <c r="E545" s="9" t="inlineStr">
@@ -60686,7 +60656,7 @@
       </c>
       <c r="D565" s="9" t="inlineStr">
         <is>
-          <t>[12443, 12582, 12333, 12477, 12570, 12400, 9003, 12422, 12399, 12321, 12491, 12623, 12231, 12245, 12393, 12430, 12379, 12514, 4332, 0, 11010, 12445, 12497, 11866, 11660, 11637, 11480, 11568, 11437, 11752, 11485]</t>
+          <t>[12447, 12586, 12337, 12481, 12574, 12404, 9006, 12426, 12403, 12325, 12495, 12627, 12235, 12249, 12397, 12434, 12383, 12518, 10223, 9723, 11501, 12449, 12502, 11870, 11664, 11641, 11483, 11571, 11441, 11756, 11489]</t>
         </is>
       </c>
     </row>
@@ -60726,7 +60696,7 @@
       </c>
       <c r="D567" s="9" t="inlineStr">
         <is>
-          <t>[12690, 12611, 12928, 12701, 12689, 12837, 12828, 12801, 12635, 12590, 12784, 12843, 12544, 12747, 12672, 12781, 12584, 12912, 12938, 2073, 709, 12711, 12714, 12643, 12610, 12910, 12871, 12722, 12784, 12829, 12641]</t>
+          <t>[12692, 12612, 12930, 12703, 12690, 12838, 12829, 12803, 12636, 12591, 12786, 12844, 12545, 12748, 12674, 12782, 12586, 12913, 12878, 9889, 10024, 12315, 12716, 12645, 12611, 12912, 12873, 12723, 12785, 12830, 12643]</t>
         </is>
       </c>
     </row>
@@ -60746,7 +60716,7 @@
       </c>
       <c r="D568" s="9" t="inlineStr">
         <is>
-          <t>[12297, 12107, 12079, 12317, 12274, 12113, 12004, 12128, 11927, 11973, 12057, 12043, 12024, 12182, 12107, 12085, 12081, 11898, 11883, 12099, 11951, 11914, 11455, 12193, 11990, 12091, 12072, 8379, 11716, 11817, 11957]</t>
+          <t>[12297, 12107, 12079, 12317, 12274, 12113, 12004, 12128, 11927, 11973, 12057, 12043, 12024, 12182, 12107, 12085, 12081, 11898, 11883, 12099, 11951, 11914, 11455, 12193, 11990, 12091, 12072, 8377, 11716, 11817, 11957]</t>
         </is>
       </c>
     </row>
@@ -60996,7 +60966,7 @@
     <row r="581">
       <c r="A581" s="9" t="inlineStr">
         <is>
-          <t>40012053</t>
+          <t>40012056</t>
         </is>
       </c>
       <c r="B581" s="9" t="inlineStr">
@@ -61055,7 +61025,7 @@
       </c>
       <c r="N581" s="9" t="inlineStr">
         <is>
-          <t>10004146</t>
+          <t>10004149</t>
         </is>
       </c>
       <c r="O581" s="9" t="n">
@@ -61071,17 +61041,17 @@
     <row r="582">
       <c r="A582" s="9" t="inlineStr">
         <is>
-          <t>40012054</t>
+          <t>40012048</t>
         </is>
       </c>
       <c r="B582" s="9" t="inlineStr">
         <is>
-          <t>PM03</t>
+          <t>PM01</t>
         </is>
       </c>
       <c r="C582" s="9" t="inlineStr">
         <is>
-          <t>PM03</t>
+          <t>PM01</t>
         </is>
       </c>
       <c r="D582" s="9" t="inlineStr">
@@ -61091,12 +61061,12 @@
       </c>
       <c r="E582" s="9" t="inlineStr">
         <is>
-          <t>LC-14</t>
+          <t>LC-04</t>
         </is>
       </c>
       <c r="F582" s="9" t="inlineStr">
         <is>
-          <t>Revisar sólidos y escala; programar tratamiento químico o el cambio de la bomba.</t>
+          <t>Reparar aislamiento del motor y del cable de LC-04</t>
         </is>
       </c>
       <c r="G582" s="9" t="inlineStr">
@@ -61105,21 +61075,21 @@
         </is>
       </c>
       <c r="H582" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I582" s="9" t="inlineStr">
         <is>
-          <t>2026-09-25T02:26:17.357+00:00</t>
+          <t>2026-09-26T19:46:00+00:00</t>
         </is>
       </c>
       <c r="J582" s="9" t="inlineStr">
         <is>
-          <t>2026-09-25T04:26:17.357+00:00</t>
+          <t>2026-09-26T20:46:00+00:00</t>
         </is>
       </c>
       <c r="K582" s="9" t="inlineStr">
         <is>
-          <t>2026-09-26T12:26:17.357+00:00</t>
+          <t>2026-09-29T10:55:00+00:00</t>
         </is>
       </c>
       <c r="L582" s="9" t="inlineStr">
@@ -61134,23 +61104,27 @@
       </c>
       <c r="N582" s="9" t="inlineStr">
         <is>
-          <t>10004147</t>
+          <t>10004148</t>
         </is>
       </c>
       <c r="O582" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="P582" s="9" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="P582" s="9" t="inlineStr">
+        <is>
+          <t>EP-LC04-260926-75</t>
+        </is>
+      </c>
       <c r="Q582" s="9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{"cantidad": 1, "material": "MAT-CAB-ESP", "descripcion": "Cable de potencia y empalme"}]</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="9" t="inlineStr">
         <is>
-          <t>40012043</t>
+          <t>40012046</t>
         </is>
       </c>
       <c r="B583" s="9" t="inlineStr">
@@ -61170,12 +61144,12 @@
       </c>
       <c r="E583" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-11</t>
         </is>
       </c>
       <c r="F583" s="9" t="inlineStr">
         <is>
-          <t>Reparar rodamientos de P-201B</t>
+          <t>Reparar aislamiento del motor y del cable de LC-11</t>
         </is>
       </c>
       <c r="G583" s="9" t="inlineStr">
@@ -61188,17 +61162,17 @@
       </c>
       <c r="I583" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22T16:05:00+00:00</t>
+          <t>2026-09-26T01:56:00+00:00</t>
         </is>
       </c>
       <c r="J583" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22T17:05:00+00:00</t>
+          <t>2026-09-26T02:56:00+00:00</t>
         </is>
       </c>
       <c r="K583" s="9" t="inlineStr">
         <is>
-          <t>2026-09-23T10:04:28+00:00</t>
+          <t>2026-09-29T16:35:00+00:00</t>
         </is>
       </c>
       <c r="L583" s="9" t="inlineStr">
@@ -61213,7 +61187,7 @@
       </c>
       <c r="N583" s="9" t="inlineStr">
         <is>
-          <t>10004143</t>
+          <t>10004146</t>
         </is>
       </c>
       <c r="O583" s="9" t="n">
@@ -61221,29 +61195,29 @@
       </c>
       <c r="P583" s="9" t="inlineStr">
         <is>
-          <t>EV-2011-0922</t>
+          <t>EP-LC11-260925-40</t>
         </is>
       </c>
       <c r="Q583" s="9" t="inlineStr">
         <is>
-          <t>[{"cantidad": 1, "material": "MAT-ROD-201", "descripcion": "Juego de rodamientos"}]</t>
+          <t>[{"cantidad": 1, "material": "MAT-CAB-ESP", "descripcion": "Cable de potencia y empalme"}]</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="9" t="inlineStr">
         <is>
-          <t>40012041</t>
+          <t>40012057</t>
         </is>
       </c>
       <c r="B584" s="9" t="inlineStr">
         <is>
-          <t>PM01</t>
+          <t>PM03</t>
         </is>
       </c>
       <c r="C584" s="9" t="inlineStr">
         <is>
-          <t>PM01</t>
+          <t>PM03</t>
         </is>
       </c>
       <c r="D584" s="9" t="inlineStr">
@@ -61253,12 +61227,12 @@
       </c>
       <c r="E584" s="9" t="inlineStr">
         <is>
-          <t>P-201B</t>
+          <t>LC-14</t>
         </is>
       </c>
       <c r="F584" s="9" t="inlineStr">
         <is>
-          <t>Reparar sello mecánico de P-201B</t>
+          <t>Revisar sólidos y escala; programar tratamiento químico o el cambio de la bomba.</t>
         </is>
       </c>
       <c r="G584" s="9" t="inlineStr">
@@ -61267,21 +61241,21 @@
         </is>
       </c>
       <c r="H584" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I584" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T03:14:00+00:00</t>
+          <t>2026-09-25T02:26:17.357+00:00</t>
         </is>
       </c>
       <c r="J584" s="9" t="inlineStr">
         <is>
-          <t>2026-09-10T04:14:00+00:00</t>
+          <t>2026-09-25T04:26:17.357+00:00</t>
         </is>
       </c>
       <c r="K584" s="9" t="inlineStr">
         <is>
-          <t>2026-09-11T15:59:36+00:00</t>
+          <t>2026-09-26T12:26:17.357+00:00</t>
         </is>
       </c>
       <c r="L584" s="9" t="inlineStr">
@@ -61296,37 +61270,33 @@
       </c>
       <c r="N584" s="9" t="inlineStr">
         <is>
-          <t>10004141</t>
+          <t>10004150</t>
         </is>
       </c>
       <c r="O584" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="P584" s="9" t="inlineStr">
-        <is>
-          <t>EV-2011-0909</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="P584" s="9" t="inlineStr"/>
       <c r="Q584" s="9" t="inlineStr">
         <is>
-          <t>[{"cantidad": 1, "material": "MAT-SELLO-201", "descripcion": "Kit de sello mecánico"}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="9" t="inlineStr">
         <is>
-          <t>40012051</t>
+          <t>40012043</t>
         </is>
       </c>
       <c r="B585" s="9" t="inlineStr">
         <is>
-          <t>PM02</t>
+          <t>PM01</t>
         </is>
       </c>
       <c r="C585" s="9" t="inlineStr">
         <is>
-          <t>PM02</t>
+          <t>PM01</t>
         </is>
       </c>
       <c r="D585" s="9" t="inlineStr">
@@ -61341,7 +61311,7 @@
       </c>
       <c r="F585" s="9" t="inlineStr">
         <is>
-          <t>Mantenimiento preventivo programado de la bomba</t>
+          <t>Reparar rodamientos de P-201B</t>
         </is>
       </c>
       <c r="G585" s="9" t="inlineStr">
@@ -61350,21 +61320,21 @@
         </is>
       </c>
       <c r="H585" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I585" s="9" t="inlineStr">
         <is>
-          <t>2026-08-12T22:49:23+00:00</t>
+          <t>2026-09-22T16:05:00+00:00</t>
         </is>
       </c>
       <c r="J585" s="9" t="inlineStr">
         <is>
-          <t>2026-08-18T22:49:23+00:00</t>
+          <t>2026-09-22T17:05:00+00:00</t>
         </is>
       </c>
       <c r="K585" s="9" t="inlineStr">
         <is>
-          <t>2026-08-20T16:34:04+00:00</t>
+          <t>2026-09-23T10:04:28+00:00</t>
         </is>
       </c>
       <c r="L585" s="9" t="inlineStr">
@@ -61377,14 +61347,22 @@
           <t>MEC-CEIBA</t>
         </is>
       </c>
-      <c r="N585" s="9" t="inlineStr"/>
+      <c r="N585" s="9" t="inlineStr">
+        <is>
+          <t>10004143</t>
+        </is>
+      </c>
       <c r="O585" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="P585" s="9" t="inlineStr"/>
+      <c r="P585" s="9" t="inlineStr">
+        <is>
+          <t>EV-2011-0922</t>
+        </is>
+      </c>
       <c r="Q585" s="9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{"cantidad": 1, "material": "MAT-ROD-201", "descripcion": "Juego de rodamientos"}]</t>
         </is>
       </c>
     </row>

</xml_diff>